<commit_message>
Resolve #53 for qpdf
</commit_message>
<xml_diff>
--- a/ISO PDF Registry.xlsx
+++ b/ISO PDF Registry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\share\pdf-names-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4646FDAD-F20F-4D0E-8D58-BE84036A32C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F712A0C-72CB-4514-8ADB-D6A31E1A5396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="29016" windowHeight="18696" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
   </bookViews>
   <sheets>
     <sheet name="PDF Prefix Registry" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="460">
   <si>
     <t>ITXT</t>
   </si>
@@ -1392,6 +1392,24 @@
   </si>
   <si>
     <t xml:space="preserve">https://github.com/adobe/pdf-names-list/issues/52 </t>
+  </si>
+  <si>
+    <t>qpdf</t>
+  </si>
+  <si>
+    <t>Manfred</t>
+  </si>
+  <si>
+    <t>Holger</t>
+  </si>
+  <si>
+    <t>manfred.holger@qpdf.org</t>
+  </si>
+  <si>
+    <t>qpdf.org</t>
+  </si>
+  <si>
+    <t>https://github.com/adobe/pdf-names-list/issues/53</t>
   </si>
 </sst>
 </file>
@@ -1808,7 +1826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E74889-C943-2949-BDAA-069F646F779D}">
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
@@ -3384,334 +3402,337 @@
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>253</v>
-      </c>
-      <c r="B76" t="s">
-        <v>254</v>
-      </c>
-      <c r="C76" t="s">
-        <v>255</v>
+      <c r="A76" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>456</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>257</v>
+        <v>457</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>458</v>
       </c>
       <c r="F76" s="5">
-        <v>44166</v>
+        <v>46038</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>104</v>
+        <v>253</v>
       </c>
       <c r="B77" t="s">
-        <v>105</v>
+        <v>254</v>
       </c>
       <c r="C77" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E77" t="s">
-        <v>108</v>
+        <v>256</v>
+      </c>
+      <c r="E77" s="8" t="s">
+        <v>257</v>
       </c>
       <c r="F77" s="5">
-        <v>41857</v>
+        <v>44166</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="B78" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="C78" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="E78" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="F78" s="5">
-        <v>42467</v>
+        <v>41857</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C79" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E79" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="F79" s="5">
-        <v>42420</v>
+        <v>42467</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>227</v>
+        <v>133</v>
       </c>
       <c r="B80" t="s">
-        <v>228</v>
+        <v>134</v>
       </c>
       <c r="C80" t="s">
-        <v>229</v>
+        <v>135</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>230</v>
+        <v>136</v>
       </c>
       <c r="E80" t="s">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="F80" s="5">
-        <v>43973</v>
+        <v>42420</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="B81" t="s">
-        <v>15</v>
+        <v>228</v>
       </c>
       <c r="C81" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="E81" t="s">
-        <v>18</v>
+        <v>231</v>
       </c>
       <c r="F81" s="5">
-        <v>40081.550694444442</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>148</v>
+        <v>14</v>
       </c>
       <c r="B82" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C82" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="E82" t="s">
-        <v>151</v>
+        <v>18</v>
       </c>
       <c r="F82" s="5">
-        <v>42472</v>
+        <v>40081.550694444442</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="B83" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C83" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E83" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="F83" s="5">
-        <v>43054</v>
+        <v>42472</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="B84" t="s">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="C84" t="s">
-        <v>301</v>
+        <v>179</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="E84" t="s">
-        <v>221</v>
+        <v>181</v>
       </c>
       <c r="F84" s="5">
-        <v>43973</v>
+        <v>43054</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="B85" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C85" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>290</v>
+        <v>220</v>
       </c>
       <c r="E85" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="F85" s="5">
-        <v>44580</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>172</v>
+        <v>288</v>
       </c>
       <c r="B86" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
       <c r="C86" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>175</v>
+        <v>290</v>
       </c>
       <c r="E86" t="s">
-        <v>176</v>
+        <v>289</v>
       </c>
       <c r="F86" s="5">
-        <v>42739</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>431</v>
+        <v>172</v>
       </c>
       <c r="B87" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C87" t="s">
-        <v>432</v>
+        <v>174</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>433</v>
+        <v>175</v>
       </c>
       <c r="E87" t="s">
-        <v>434</v>
+        <v>176</v>
       </c>
       <c r="F87" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G87" s="1" t="s">
-        <v>435</v>
+        <v>42739</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>375</v>
+        <v>431</v>
       </c>
       <c r="B88" t="s">
-        <v>376</v>
+        <v>183</v>
       </c>
       <c r="C88" t="s">
-        <v>377</v>
+        <v>432</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="E88" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="F88" s="5">
-        <v>45358</v>
+        <v>45818</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>39</v>
+        <v>375</v>
       </c>
       <c r="B89" t="s">
-        <v>40</v>
+        <v>376</v>
       </c>
       <c r="C89" t="s">
-        <v>41</v>
+        <v>377</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>42</v>
+        <v>378</v>
       </c>
       <c r="E89" t="s">
-        <v>43</v>
+        <v>379</v>
       </c>
       <c r="F89" s="5">
-        <v>40522.519444444442</v>
+        <v>45358</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="B90" t="s">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="C90" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="E90" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="F90" s="5">
-        <v>41890</v>
+        <v>40522.519444444442</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="B91" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="C91" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="E91" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="F91" s="5">
-        <v>42852</v>
+        <v>41890</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>177</v>
+        <v>64</v>
       </c>
       <c r="B92" t="s">
         <v>65</v>
@@ -3731,104 +3752,124 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B93" t="s">
-        <v>204</v>
+        <v>65</v>
       </c>
       <c r="C93" t="s">
-        <v>205</v>
+        <v>66</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="F93" s="6">
-        <v>43487</v>
+        <v>67</v>
+      </c>
+      <c r="E93" t="s">
+        <v>68</v>
+      </c>
+      <c r="F93" s="5">
+        <v>42852</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="B94" t="s">
-        <v>157</v>
+        <v>204</v>
       </c>
       <c r="C94" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E94" t="s">
-        <v>160</v>
-      </c>
-      <c r="F94" s="5">
-        <v>42505</v>
+        <v>206</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F94" s="6">
+        <v>43487</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>409</v>
+        <v>156</v>
       </c>
       <c r="B95" t="s">
-        <v>361</v>
+        <v>157</v>
       </c>
       <c r="C95" t="s">
-        <v>362</v>
+        <v>158</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>363</v>
+        <v>159</v>
       </c>
       <c r="E95" t="s">
-        <v>214</v>
+        <v>160</v>
       </c>
       <c r="F95" s="5">
-        <v>45695</v>
-      </c>
-      <c r="G95" t="s">
-        <v>410</v>
+        <v>42505</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>329</v>
+        <v>409</v>
       </c>
       <c r="B96" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C96" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="E96" t="s">
-        <v>333</v>
+        <v>214</v>
       </c>
       <c r="F96" s="5">
-        <v>44775</v>
+        <v>45695</v>
+      </c>
+      <c r="G96" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
+        <v>329</v>
+      </c>
+      <c r="B97" t="s">
+        <v>330</v>
+      </c>
+      <c r="C97" t="s">
+        <v>331</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E97" t="s">
+        <v>333</v>
+      </c>
+      <c r="F97" s="5">
+        <v>44775</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
         <v>138</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B98" t="s">
         <v>139</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C98" t="s">
         <v>140</v>
       </c>
-      <c r="D97" s="1" t="s">
+      <c r="D98" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E98" t="s">
         <v>142</v>
       </c>
-      <c r="F97" s="5">
+      <c r="F98" s="5">
         <v>42439</v>
       </c>
     </row>
@@ -3844,41 +3885,41 @@
     <hyperlink ref="D57" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
     <hyperlink ref="D49" r:id="rId4" xr:uid="{234AD513-3ABE-F545-A037-27824EABDF68}"/>
     <hyperlink ref="D41" r:id="rId5" xr:uid="{7924D455-5B5F-E641-AB7C-FB4BD03EF051}"/>
-    <hyperlink ref="D80" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
+    <hyperlink ref="D81" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
     <hyperlink ref="D40" r:id="rId7" xr:uid="{7AEF03BC-D893-FF42-BB52-AB9C9480EA0D}"/>
-    <hyperlink ref="D84" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
+    <hyperlink ref="D85" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
     <hyperlink ref="D12" r:id="rId9" xr:uid="{D57F2423-845A-9E44-A60D-DEEB1150BE7A}"/>
     <hyperlink ref="D10" r:id="rId10" xr:uid="{0133BED0-2D2B-4A0F-AB7C-D58D8B5F381B}"/>
     <hyperlink ref="D3" r:id="rId11" xr:uid="{5F0875F3-1434-4B08-A87A-2BDF5EEDDAC9}"/>
     <hyperlink ref="D26" r:id="rId12" xr:uid="{61482C13-D6B2-4AFF-AD10-908ABE8BA3F2}"/>
-    <hyperlink ref="D76" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
+    <hyperlink ref="D77" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
     <hyperlink ref="D47" r:id="rId14" xr:uid="{FEB07F00-70C8-4D84-B7DF-B36DF7C6138C}"/>
     <hyperlink ref="D36" r:id="rId15" xr:uid="{9236AFAC-B489-4804-B65A-1988399CC4C2}"/>
     <hyperlink ref="D75" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
-    <hyperlink ref="D93" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
+    <hyperlink ref="D94" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
     <hyperlink ref="D74" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
     <hyperlink ref="D30" r:id="rId19" xr:uid="{178F076F-6CAC-44EB-AA97-31037608AA41}"/>
     <hyperlink ref="D38" r:id="rId20" xr:uid="{E467E97B-65A6-40E0-A2BA-7875E3A5C2C1}"/>
-    <hyperlink ref="D83" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
-    <hyperlink ref="D92" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
-    <hyperlink ref="D86" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
+    <hyperlink ref="D84" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
+    <hyperlink ref="D93" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
+    <hyperlink ref="D87" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
     <hyperlink ref="D17" r:id="rId24" xr:uid="{8C069B77-F7A2-4DC6-9D5A-D5138E5E1158}"/>
     <hyperlink ref="D16" r:id="rId25" xr:uid="{C770D7DE-6980-45A2-A8B6-8E4C376C05E3}"/>
     <hyperlink ref="D69" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
-    <hyperlink ref="D94" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
+    <hyperlink ref="D95" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
     <hyperlink ref="D50" r:id="rId28" xr:uid="{2B927B9E-56D2-4AC7-A24B-BA7FAF44F900}"/>
     <hyperlink ref="D33" r:id="rId29" xr:uid="{5F9DAD98-7221-4BEC-B311-BF6B1BD6F52E}"/>
-    <hyperlink ref="D81" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
+    <hyperlink ref="D82" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
     <hyperlink ref="D51" r:id="rId31" xr:uid="{7BC6DF64-9FBB-461B-BEE3-D705D5A5711D}"/>
     <hyperlink ref="D21" r:id="rId32" xr:uid="{EE5546A8-9D18-43D6-949A-451AA8A97E76}"/>
     <hyperlink ref="D71" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
     <hyperlink ref="D42" r:id="rId34" xr:uid="{03938AC4-898D-4B60-9A83-CF770912371F}"/>
-    <hyperlink ref="D89" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
+    <hyperlink ref="D90" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
     <hyperlink ref="D62" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
     <hyperlink ref="D7" r:id="rId37" xr:uid="{C501338A-FD0F-4F45-B8B1-BD737635609F}"/>
     <hyperlink ref="D37" r:id="rId38" xr:uid="{973F790E-4686-49DC-8382-D85663F42FE4}"/>
     <hyperlink ref="D55" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
-    <hyperlink ref="D91" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
+    <hyperlink ref="D92" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
     <hyperlink ref="D13" r:id="rId41" xr:uid="{E0321D7C-4A33-425C-AC81-F2844EF49280}"/>
     <hyperlink ref="D44" r:id="rId42" xr:uid="{9362C2F6-92F8-4578-90F4-F93A12DB0620}"/>
     <hyperlink ref="D48" r:id="rId43" xr:uid="{3D2507DB-58F1-46EB-972C-7262C11F3BC0}"/>
@@ -3886,22 +3927,22 @@
     <hyperlink ref="D68" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
     <hyperlink ref="D52" r:id="rId46" xr:uid="{FA35DE19-FE12-4948-8782-601512787A1F}"/>
     <hyperlink ref="D73" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
-    <hyperlink ref="D77" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
-    <hyperlink ref="D90" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
+    <hyperlink ref="D78" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
+    <hyperlink ref="D91" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
     <hyperlink ref="D60" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
     <hyperlink ref="D27" r:id="rId51" xr:uid="{20CCBF4F-DA07-40B1-84D7-9C64B10A18DD}"/>
     <hyperlink ref="D4" r:id="rId52" xr:uid="{04F40983-3CCF-4A98-9D71-83239E621071}"/>
     <hyperlink ref="D32" r:id="rId53" xr:uid="{B6182D1F-82B7-4DC3-BB62-5D4CE3E6347D}"/>
-    <hyperlink ref="D79" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
-    <hyperlink ref="D97" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
-    <hyperlink ref="D78" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
-    <hyperlink ref="D82" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
+    <hyperlink ref="D80" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
+    <hyperlink ref="D98" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
+    <hyperlink ref="D79" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
+    <hyperlink ref="D83" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
     <hyperlink ref="D9" r:id="rId58" xr:uid="{F7E14BE7-9BEF-429A-BC06-CA914EDCD03E}"/>
     <hyperlink ref="D23" r:id="rId59" xr:uid="{13F0A7EA-4265-4C1A-936D-0F1F22648B66}"/>
     <hyperlink ref="D43" r:id="rId60" display="mailto:david@zwang.com" xr:uid="{2E031ABA-CF1B-48A8-96E6-B6DCE94345AE}"/>
     <hyperlink ref="D65" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
     <hyperlink ref="D66" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
-    <hyperlink ref="D85" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
+    <hyperlink ref="D86" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
     <hyperlink ref="D29" r:id="rId64" xr:uid="{3AD048BB-9D70-41FA-8645-47CF1BE084C9}"/>
     <hyperlink ref="D31" r:id="rId65" display="mailto:bertvk@enfocus.com" xr:uid="{6F56AFA2-CA54-4A51-B51B-36740F243F7A}"/>
     <hyperlink ref="D46" r:id="rId66" xr:uid="{DEECD580-BF33-4FBB-A267-48E6674FF044}"/>
@@ -3909,7 +3950,7 @@
     <hyperlink ref="D19" r:id="rId68" xr:uid="{897A4DB8-756C-42E5-AF7B-011BBBE00628}"/>
     <hyperlink ref="D39" r:id="rId69" xr:uid="{47A4E692-159B-4E48-A1D4-411E278B3A43}"/>
     <hyperlink ref="D2" r:id="rId70" display="mailto:frank.vyncke@yin4yang.com" xr:uid="{E29600CB-349C-4C55-AC29-3B61912C4757}"/>
-    <hyperlink ref="D96" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
+    <hyperlink ref="D97" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
     <hyperlink ref="D25" r:id="rId72" xr:uid="{BF5FD244-0DE0-493E-A7E1-0CEDCE9B77AA}"/>
     <hyperlink ref="D5" r:id="rId73" xr:uid="{33D12C26-CC5E-4925-86B6-4AE855A6371F}"/>
     <hyperlink ref="G5" r:id="rId74" xr:uid="{2FA39695-7884-42EC-9380-C8EFD7B7EAD9}"/>
@@ -3922,8 +3963,8 @@
     <hyperlink ref="D63" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
     <hyperlink ref="D45" r:id="rId82" xr:uid="{72B2BA10-0B55-4ACF-9CC1-DA30FB4C2741}"/>
     <hyperlink ref="G45" r:id="rId83" xr:uid="{1106BFBB-F6F3-4E8A-8B65-06381130271C}"/>
-    <hyperlink ref="D88" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
-    <hyperlink ref="G88" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
+    <hyperlink ref="D89" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
+    <hyperlink ref="G89" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
     <hyperlink ref="G53" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
     <hyperlink ref="D53" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
     <hyperlink ref="G20" r:id="rId88" xr:uid="{C64F139E-8286-4E7A-8B5E-9D69FC9A0C25}"/>
@@ -3935,7 +3976,7 @@
     <hyperlink ref="D35" r:id="rId94" xr:uid="{F07464A9-7B4E-4E5B-9EEE-3F687E9DC9AC}"/>
     <hyperlink ref="G35" r:id="rId95" xr:uid="{73C68A69-730D-4676-B564-01BC2FDA7E73}"/>
     <hyperlink ref="D67" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
-    <hyperlink ref="D95" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
+    <hyperlink ref="D96" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
     <hyperlink ref="D22" r:id="rId98" xr:uid="{3C768ED5-B6E7-416A-B3CF-31E9B14F1258}"/>
     <hyperlink ref="G22" r:id="rId99" xr:uid="{5C4AC9BE-92AA-40F8-AA34-D54E19486DEE}"/>
     <hyperlink ref="D8" r:id="rId100" xr:uid="{0DDFD3D5-41E0-4A59-8992-A1EE6FD3C05D}"/>
@@ -3944,16 +3985,18 @@
     <hyperlink ref="G72" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
     <hyperlink ref="G61" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
     <hyperlink ref="D61" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
-    <hyperlink ref="D87" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
-    <hyperlink ref="G87" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
+    <hyperlink ref="D88" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
+    <hyperlink ref="G88" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
     <hyperlink ref="D54" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
     <hyperlink ref="G54" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
     <hyperlink ref="D24" r:id="rId110" xr:uid="{42EF2DCB-F6A9-4EC5-9C1C-9B9A137FDD6C}"/>
     <hyperlink ref="G24" r:id="rId111" xr:uid="{68016CF6-F4CA-4852-AF56-7954DB739663}"/>
     <hyperlink ref="D58" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
     <hyperlink ref="G58" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
+    <hyperlink ref="D76" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
+    <hyperlink ref="G76" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId114"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId116"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve PXCE (Issue #54)
</commit_message>
<xml_diff>
--- a/ISO PDF Registry.xlsx
+++ b/ISO PDF Registry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\share\pdf-names-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F712A0C-72CB-4514-8ADB-D6A31E1A5396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0F7479-BFCA-49A3-BA79-411D39DBFEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
+    <workbookView xWindow="-34740" yWindow="3660" windowWidth="28800" windowHeight="15285" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
   </bookViews>
   <sheets>
     <sheet name="PDF Prefix Registry" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="466">
   <si>
     <t>ITXT</t>
   </si>
@@ -1410,6 +1410,24 @@
   </si>
   <si>
     <t>https://github.com/adobe/pdf-names-list/issues/53</t>
+  </si>
+  <si>
+    <t>PXCE</t>
+  </si>
+  <si>
+    <t>Ivan</t>
+  </si>
+  <si>
+    <t>Poberezhnyk</t>
+  </si>
+  <si>
+    <t>ivan@pdf-xchange.com</t>
+  </si>
+  <si>
+    <t>PDF-XChange Co Ltd.</t>
+  </si>
+  <si>
+    <t>https://github.com/adobe/pdf-names-list/issues/54</t>
   </si>
 </sst>
 </file>
@@ -1826,7 +1844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E74889-C943-2949-BDAA-069F646F779D}">
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
@@ -3403,356 +3421,359 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="C76" t="s">
+        <v>462</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="E76" t="s">
+        <v>464</v>
+      </c>
+      <c r="F76" s="5">
+        <v>46090</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B77" s="7" t="s">
         <v>455</v>
       </c>
-      <c r="C76" s="7" t="s">
+      <c r="C77" s="7" t="s">
         <v>456</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="D77" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E76" s="7" t="s">
+      <c r="E77" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="F76" s="5">
+      <c r="F77" s="5">
         <v>46038</v>
       </c>
-      <c r="G76" s="1" t="s">
+      <c r="G77" s="1" t="s">
         <v>459</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>253</v>
-      </c>
-      <c r="B77" t="s">
-        <v>254</v>
-      </c>
-      <c r="C77" t="s">
-        <v>255</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E77" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="F77" s="5">
-        <v>44166</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>104</v>
+        <v>253</v>
       </c>
       <c r="B78" t="s">
-        <v>105</v>
+        <v>254</v>
       </c>
       <c r="C78" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E78" t="s">
-        <v>108</v>
+        <v>256</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>257</v>
       </c>
       <c r="F78" s="5">
-        <v>41857</v>
+        <v>44166</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="B79" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="C79" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="E79" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="F79" s="5">
-        <v>42467</v>
+        <v>41857</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B80" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C80" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E80" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="F80" s="5">
-        <v>42420</v>
+        <v>42467</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>227</v>
+        <v>133</v>
       </c>
       <c r="B81" t="s">
-        <v>228</v>
+        <v>134</v>
       </c>
       <c r="C81" t="s">
-        <v>229</v>
+        <v>135</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>230</v>
+        <v>136</v>
       </c>
       <c r="E81" t="s">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="F81" s="5">
-        <v>43973</v>
+        <v>42420</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="B82" t="s">
-        <v>15</v>
+        <v>228</v>
       </c>
       <c r="C82" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="E82" t="s">
-        <v>18</v>
+        <v>231</v>
       </c>
       <c r="F82" s="5">
-        <v>40081.550694444442</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>148</v>
+        <v>14</v>
       </c>
       <c r="B83" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C83" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="E83" t="s">
-        <v>151</v>
+        <v>18</v>
       </c>
       <c r="F83" s="5">
-        <v>42472</v>
+        <v>40081.550694444442</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="B84" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C84" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E84" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="F84" s="5">
-        <v>43054</v>
+        <v>42472</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="B85" t="s">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="C85" t="s">
-        <v>301</v>
+        <v>179</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="E85" t="s">
-        <v>221</v>
+        <v>181</v>
       </c>
       <c r="F85" s="5">
-        <v>43973</v>
+        <v>43054</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="B86" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C86" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>290</v>
+        <v>220</v>
       </c>
       <c r="E86" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="F86" s="5">
-        <v>44580</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>172</v>
+        <v>288</v>
       </c>
       <c r="B87" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
       <c r="C87" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>175</v>
+        <v>290</v>
       </c>
       <c r="E87" t="s">
-        <v>176</v>
+        <v>289</v>
       </c>
       <c r="F87" s="5">
-        <v>42739</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>431</v>
+        <v>172</v>
       </c>
       <c r="B88" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C88" t="s">
-        <v>432</v>
+        <v>174</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>433</v>
+        <v>175</v>
       </c>
       <c r="E88" t="s">
-        <v>434</v>
+        <v>176</v>
       </c>
       <c r="F88" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G88" s="1" t="s">
-        <v>435</v>
+        <v>42739</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>375</v>
+        <v>431</v>
       </c>
       <c r="B89" t="s">
-        <v>376</v>
+        <v>183</v>
       </c>
       <c r="C89" t="s">
-        <v>377</v>
+        <v>432</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="E89" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="F89" s="5">
-        <v>45358</v>
+        <v>45818</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>39</v>
+        <v>375</v>
       </c>
       <c r="B90" t="s">
-        <v>40</v>
+        <v>376</v>
       </c>
       <c r="C90" t="s">
-        <v>41</v>
+        <v>377</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>42</v>
+        <v>378</v>
       </c>
       <c r="E90" t="s">
-        <v>43</v>
+        <v>379</v>
       </c>
       <c r="F90" s="5">
-        <v>40522.519444444442</v>
+        <v>45358</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="B91" t="s">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="E91" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="F91" s="5">
-        <v>41890</v>
+        <v>40522.519444444442</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="B92" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="C92" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="E92" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="F92" s="5">
-        <v>42852</v>
+        <v>41890</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>177</v>
+        <v>64</v>
       </c>
       <c r="B93" t="s">
         <v>65</v>
@@ -3772,104 +3793,124 @@
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B94" t="s">
-        <v>204</v>
+        <v>65</v>
       </c>
       <c r="C94" t="s">
-        <v>205</v>
+        <v>66</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="F94" s="6">
-        <v>43487</v>
+        <v>67</v>
+      </c>
+      <c r="E94" t="s">
+        <v>68</v>
+      </c>
+      <c r="F94" s="5">
+        <v>42852</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="B95" t="s">
-        <v>157</v>
+        <v>204</v>
       </c>
       <c r="C95" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E95" t="s">
-        <v>160</v>
-      </c>
-      <c r="F95" s="5">
-        <v>42505</v>
+        <v>206</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F95" s="6">
+        <v>43487</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
+        <v>156</v>
+      </c>
+      <c r="B96" t="s">
+        <v>157</v>
+      </c>
+      <c r="C96" t="s">
+        <v>158</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E96" t="s">
+        <v>160</v>
+      </c>
+      <c r="F96" s="5">
+        <v>42505</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>409</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B97" t="s">
         <v>361</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C97" t="s">
         <v>362</v>
       </c>
-      <c r="D96" s="1" t="s">
+      <c r="D97" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E97" t="s">
         <v>214</v>
       </c>
-      <c r="F96" s="5">
+      <c r="F97" s="5">
         <v>45695</v>
       </c>
-      <c r="G96" t="s">
+      <c r="G97" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
         <v>329</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B98" t="s">
         <v>330</v>
       </c>
-      <c r="C97" t="s">
+      <c r="C98" t="s">
         <v>331</v>
       </c>
-      <c r="D97" s="1" t="s">
+      <c r="D98" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E98" t="s">
         <v>333</v>
       </c>
-      <c r="F97" s="5">
+      <c r="F98" s="5">
         <v>44775</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
         <v>138</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B99" t="s">
         <v>139</v>
       </c>
-      <c r="C98" t="s">
+      <c r="C99" t="s">
         <v>140</v>
       </c>
-      <c r="D98" s="1" t="s">
+      <c r="D99" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E98" t="s">
+      <c r="E99" t="s">
         <v>142</v>
       </c>
-      <c r="F98" s="5">
+      <c r="F99" s="5">
         <v>42439</v>
       </c>
     </row>
@@ -3885,41 +3926,41 @@
     <hyperlink ref="D57" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
     <hyperlink ref="D49" r:id="rId4" xr:uid="{234AD513-3ABE-F545-A037-27824EABDF68}"/>
     <hyperlink ref="D41" r:id="rId5" xr:uid="{7924D455-5B5F-E641-AB7C-FB4BD03EF051}"/>
-    <hyperlink ref="D81" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
+    <hyperlink ref="D82" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
     <hyperlink ref="D40" r:id="rId7" xr:uid="{7AEF03BC-D893-FF42-BB52-AB9C9480EA0D}"/>
-    <hyperlink ref="D85" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
+    <hyperlink ref="D86" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
     <hyperlink ref="D12" r:id="rId9" xr:uid="{D57F2423-845A-9E44-A60D-DEEB1150BE7A}"/>
     <hyperlink ref="D10" r:id="rId10" xr:uid="{0133BED0-2D2B-4A0F-AB7C-D58D8B5F381B}"/>
     <hyperlink ref="D3" r:id="rId11" xr:uid="{5F0875F3-1434-4B08-A87A-2BDF5EEDDAC9}"/>
     <hyperlink ref="D26" r:id="rId12" xr:uid="{61482C13-D6B2-4AFF-AD10-908ABE8BA3F2}"/>
-    <hyperlink ref="D77" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
+    <hyperlink ref="D78" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
     <hyperlink ref="D47" r:id="rId14" xr:uid="{FEB07F00-70C8-4D84-B7DF-B36DF7C6138C}"/>
     <hyperlink ref="D36" r:id="rId15" xr:uid="{9236AFAC-B489-4804-B65A-1988399CC4C2}"/>
     <hyperlink ref="D75" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
-    <hyperlink ref="D94" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
+    <hyperlink ref="D95" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
     <hyperlink ref="D74" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
     <hyperlink ref="D30" r:id="rId19" xr:uid="{178F076F-6CAC-44EB-AA97-31037608AA41}"/>
     <hyperlink ref="D38" r:id="rId20" xr:uid="{E467E97B-65A6-40E0-A2BA-7875E3A5C2C1}"/>
-    <hyperlink ref="D84" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
-    <hyperlink ref="D93" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
-    <hyperlink ref="D87" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
+    <hyperlink ref="D85" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
+    <hyperlink ref="D94" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
+    <hyperlink ref="D88" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
     <hyperlink ref="D17" r:id="rId24" xr:uid="{8C069B77-F7A2-4DC6-9D5A-D5138E5E1158}"/>
     <hyperlink ref="D16" r:id="rId25" xr:uid="{C770D7DE-6980-45A2-A8B6-8E4C376C05E3}"/>
     <hyperlink ref="D69" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
-    <hyperlink ref="D95" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
+    <hyperlink ref="D96" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
     <hyperlink ref="D50" r:id="rId28" xr:uid="{2B927B9E-56D2-4AC7-A24B-BA7FAF44F900}"/>
     <hyperlink ref="D33" r:id="rId29" xr:uid="{5F9DAD98-7221-4BEC-B311-BF6B1BD6F52E}"/>
-    <hyperlink ref="D82" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
+    <hyperlink ref="D83" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
     <hyperlink ref="D51" r:id="rId31" xr:uid="{7BC6DF64-9FBB-461B-BEE3-D705D5A5711D}"/>
     <hyperlink ref="D21" r:id="rId32" xr:uid="{EE5546A8-9D18-43D6-949A-451AA8A97E76}"/>
     <hyperlink ref="D71" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
     <hyperlink ref="D42" r:id="rId34" xr:uid="{03938AC4-898D-4B60-9A83-CF770912371F}"/>
-    <hyperlink ref="D90" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
+    <hyperlink ref="D91" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
     <hyperlink ref="D62" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
     <hyperlink ref="D7" r:id="rId37" xr:uid="{C501338A-FD0F-4F45-B8B1-BD737635609F}"/>
     <hyperlink ref="D37" r:id="rId38" xr:uid="{973F790E-4686-49DC-8382-D85663F42FE4}"/>
     <hyperlink ref="D55" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
-    <hyperlink ref="D92" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
+    <hyperlink ref="D93" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
     <hyperlink ref="D13" r:id="rId41" xr:uid="{E0321D7C-4A33-425C-AC81-F2844EF49280}"/>
     <hyperlink ref="D44" r:id="rId42" xr:uid="{9362C2F6-92F8-4578-90F4-F93A12DB0620}"/>
     <hyperlink ref="D48" r:id="rId43" xr:uid="{3D2507DB-58F1-46EB-972C-7262C11F3BC0}"/>
@@ -3927,22 +3968,22 @@
     <hyperlink ref="D68" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
     <hyperlink ref="D52" r:id="rId46" xr:uid="{FA35DE19-FE12-4948-8782-601512787A1F}"/>
     <hyperlink ref="D73" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
-    <hyperlink ref="D78" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
-    <hyperlink ref="D91" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
+    <hyperlink ref="D79" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
+    <hyperlink ref="D92" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
     <hyperlink ref="D60" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
     <hyperlink ref="D27" r:id="rId51" xr:uid="{20CCBF4F-DA07-40B1-84D7-9C64B10A18DD}"/>
     <hyperlink ref="D4" r:id="rId52" xr:uid="{04F40983-3CCF-4A98-9D71-83239E621071}"/>
     <hyperlink ref="D32" r:id="rId53" xr:uid="{B6182D1F-82B7-4DC3-BB62-5D4CE3E6347D}"/>
-    <hyperlink ref="D80" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
-    <hyperlink ref="D98" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
-    <hyperlink ref="D79" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
-    <hyperlink ref="D83" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
+    <hyperlink ref="D81" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
+    <hyperlink ref="D99" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
+    <hyperlink ref="D80" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
+    <hyperlink ref="D84" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
     <hyperlink ref="D9" r:id="rId58" xr:uid="{F7E14BE7-9BEF-429A-BC06-CA914EDCD03E}"/>
     <hyperlink ref="D23" r:id="rId59" xr:uid="{13F0A7EA-4265-4C1A-936D-0F1F22648B66}"/>
     <hyperlink ref="D43" r:id="rId60" display="mailto:david@zwang.com" xr:uid="{2E031ABA-CF1B-48A8-96E6-B6DCE94345AE}"/>
     <hyperlink ref="D65" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
     <hyperlink ref="D66" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
-    <hyperlink ref="D86" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
+    <hyperlink ref="D87" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
     <hyperlink ref="D29" r:id="rId64" xr:uid="{3AD048BB-9D70-41FA-8645-47CF1BE084C9}"/>
     <hyperlink ref="D31" r:id="rId65" display="mailto:bertvk@enfocus.com" xr:uid="{6F56AFA2-CA54-4A51-B51B-36740F243F7A}"/>
     <hyperlink ref="D46" r:id="rId66" xr:uid="{DEECD580-BF33-4FBB-A267-48E6674FF044}"/>
@@ -3950,7 +3991,7 @@
     <hyperlink ref="D19" r:id="rId68" xr:uid="{897A4DB8-756C-42E5-AF7B-011BBBE00628}"/>
     <hyperlink ref="D39" r:id="rId69" xr:uid="{47A4E692-159B-4E48-A1D4-411E278B3A43}"/>
     <hyperlink ref="D2" r:id="rId70" display="mailto:frank.vyncke@yin4yang.com" xr:uid="{E29600CB-349C-4C55-AC29-3B61912C4757}"/>
-    <hyperlink ref="D97" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
+    <hyperlink ref="D98" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
     <hyperlink ref="D25" r:id="rId72" xr:uid="{BF5FD244-0DE0-493E-A7E1-0CEDCE9B77AA}"/>
     <hyperlink ref="D5" r:id="rId73" xr:uid="{33D12C26-CC5E-4925-86B6-4AE855A6371F}"/>
     <hyperlink ref="G5" r:id="rId74" xr:uid="{2FA39695-7884-42EC-9380-C8EFD7B7EAD9}"/>
@@ -3963,8 +4004,8 @@
     <hyperlink ref="D63" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
     <hyperlink ref="D45" r:id="rId82" xr:uid="{72B2BA10-0B55-4ACF-9CC1-DA30FB4C2741}"/>
     <hyperlink ref="G45" r:id="rId83" xr:uid="{1106BFBB-F6F3-4E8A-8B65-06381130271C}"/>
-    <hyperlink ref="D89" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
-    <hyperlink ref="G89" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
+    <hyperlink ref="D90" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
+    <hyperlink ref="G90" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
     <hyperlink ref="G53" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
     <hyperlink ref="D53" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
     <hyperlink ref="G20" r:id="rId88" xr:uid="{C64F139E-8286-4E7A-8B5E-9D69FC9A0C25}"/>
@@ -3976,7 +4017,7 @@
     <hyperlink ref="D35" r:id="rId94" xr:uid="{F07464A9-7B4E-4E5B-9EEE-3F687E9DC9AC}"/>
     <hyperlink ref="G35" r:id="rId95" xr:uid="{73C68A69-730D-4676-B564-01BC2FDA7E73}"/>
     <hyperlink ref="D67" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
-    <hyperlink ref="D96" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
+    <hyperlink ref="D97" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
     <hyperlink ref="D22" r:id="rId98" xr:uid="{3C768ED5-B6E7-416A-B3CF-31E9B14F1258}"/>
     <hyperlink ref="G22" r:id="rId99" xr:uid="{5C4AC9BE-92AA-40F8-AA34-D54E19486DEE}"/>
     <hyperlink ref="D8" r:id="rId100" xr:uid="{0DDFD3D5-41E0-4A59-8992-A1EE6FD3C05D}"/>
@@ -3985,18 +4026,19 @@
     <hyperlink ref="G72" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
     <hyperlink ref="G61" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
     <hyperlink ref="D61" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
-    <hyperlink ref="D88" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
-    <hyperlink ref="G88" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
+    <hyperlink ref="D89" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
+    <hyperlink ref="G89" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
     <hyperlink ref="D54" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
     <hyperlink ref="G54" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
     <hyperlink ref="D24" r:id="rId110" xr:uid="{42EF2DCB-F6A9-4EC5-9C1C-9B9A137FDD6C}"/>
     <hyperlink ref="G24" r:id="rId111" xr:uid="{68016CF6-F4CA-4852-AF56-7954DB739663}"/>
     <hyperlink ref="D58" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
     <hyperlink ref="G58" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
-    <hyperlink ref="D76" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
-    <hyperlink ref="G76" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
+    <hyperlink ref="D77" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
+    <hyperlink ref="G77" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
+    <hyperlink ref="G76" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId116"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId117"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Note mistake in ESTI 319 142-1 referring to ESIX instead of ESIC
</commit_message>
<xml_diff>
--- a/ISO PDF Registry.xlsx
+++ b/ISO PDF Registry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\share\pdf-names-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0F7479-BFCA-49A3-BA79-411D39DBFEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55F86DA-F28C-4181-97BA-C5FB8BC31C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-34740" yWindow="3660" windowWidth="28800" windowHeight="15285" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="469">
   <si>
     <t>ITXT</t>
   </si>
@@ -1428,6 +1428,15 @@
   </si>
   <si>
     <t>https://github.com/adobe/pdf-names-list/issues/54</t>
+  </si>
+  <si>
+    <t>ESIX</t>
+  </si>
+  <si>
+    <t>ETSI EN 319 142-2 V1.2.1 (2025-07) mentions ESIX with reference to ETSI EN 319 142-1, but 319 142-1 only uses ESIC. Thus ESIX is considered a typographic error.</t>
+  </si>
+  <si>
+    <t>ETSI Electronic Signatures and Infrastructures Committee (for PAdES) - DO NOT USE THIS PREFIX - use ESIC</t>
   </si>
 </sst>
 </file>
@@ -1437,7 +1446,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1482,6 +1491,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1513,7 +1528,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1529,6 +1544,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1844,14 +1860,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E74889-C943-2949-BDAA-069F646F779D}">
-  <dimension ref="A1:G99"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
     <col min="2" max="2" width="16.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.8984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="83.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="90.69921875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.8984375" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="44.296875" bestFit="1" customWidth="1"/>
   </cols>
@@ -2451,774 +2467,777 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>293</v>
+        <v>466</v>
       </c>
       <c r="B29" t="s">
-        <v>296</v>
+        <v>399</v>
       </c>
       <c r="C29" t="s">
-        <v>297</v>
+        <v>400</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>295</v>
+        <v>401</v>
       </c>
       <c r="E29" t="s">
-        <v>294</v>
+        <v>468</v>
       </c>
       <c r="F29" s="5">
-        <v>44580</v>
-      </c>
-      <c r="G29" t="s">
-        <v>299</v>
+        <v>46090</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>187</v>
+        <v>293</v>
       </c>
       <c r="B30" t="s">
-        <v>188</v>
+        <v>296</v>
       </c>
       <c r="C30" t="s">
-        <v>189</v>
+        <v>297</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>190</v>
+        <v>295</v>
       </c>
       <c r="E30" t="s">
-        <v>191</v>
+        <v>294</v>
       </c>
       <c r="F30" s="5">
-        <v>43231</v>
+        <v>44580</v>
+      </c>
+      <c r="G30" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>303</v>
+        <v>187</v>
       </c>
       <c r="B31" t="s">
-        <v>304</v>
+        <v>188</v>
       </c>
       <c r="C31" t="s">
-        <v>305</v>
+        <v>189</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>306</v>
+        <v>190</v>
       </c>
       <c r="E31" t="s">
-        <v>307</v>
+        <v>191</v>
       </c>
       <c r="F31" s="5">
-        <v>44581</v>
-      </c>
-      <c r="G31" t="s">
-        <v>299</v>
+        <v>43231</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>128</v>
+        <v>303</v>
       </c>
       <c r="B32" t="s">
-        <v>129</v>
+        <v>304</v>
       </c>
       <c r="C32" t="s">
-        <v>130</v>
+        <v>305</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>131</v>
+        <v>306</v>
       </c>
       <c r="E32" t="s">
-        <v>132</v>
+        <v>307</v>
       </c>
       <c r="F32" s="5">
-        <v>41680</v>
+        <v>44581</v>
+      </c>
+      <c r="G32" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>128</v>
       </c>
       <c r="B33" t="s">
-        <v>10</v>
+        <v>129</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>130</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>12</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>13</v>
+        <v>132</v>
       </c>
       <c r="F33" s="5">
-        <v>40079.444444444445</v>
+        <v>41680</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>321</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
-        <v>209</v>
+        <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>210</v>
+        <v>11</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>322</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>323</v>
+        <v>13</v>
       </c>
       <c r="F34" s="5">
-        <v>44774</v>
+        <v>40079.444444444445</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>402</v>
+        <v>321</v>
       </c>
       <c r="B35" t="s">
-        <v>403</v>
+        <v>209</v>
       </c>
       <c r="C35" t="s">
-        <v>404</v>
+        <v>210</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>405</v>
+        <v>322</v>
       </c>
       <c r="E35" t="s">
-        <v>406</v>
+        <v>323</v>
       </c>
       <c r="F35" s="5">
-        <v>45673</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>407</v>
+        <v>44774</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>244</v>
+        <v>402</v>
       </c>
       <c r="B36" t="s">
-        <v>173</v>
+        <v>403</v>
       </c>
       <c r="C36" t="s">
-        <v>245</v>
+        <v>404</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>246</v>
+        <v>405</v>
       </c>
       <c r="E36" t="s">
-        <v>247</v>
+        <v>406</v>
       </c>
       <c r="F36" s="5">
-        <v>44037</v>
+        <v>45673</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>53</v>
+        <v>244</v>
       </c>
       <c r="B37" t="s">
-        <v>54</v>
+        <v>173</v>
       </c>
       <c r="C37" t="s">
-        <v>54</v>
+        <v>245</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>55</v>
+        <v>246</v>
       </c>
       <c r="E37" t="s">
-        <v>56</v>
+        <v>247</v>
       </c>
       <c r="F37" s="5">
-        <v>40714.365972222222</v>
+        <v>44037</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>182</v>
+        <v>53</v>
       </c>
       <c r="B38" t="s">
-        <v>183</v>
+        <v>54</v>
       </c>
       <c r="C38" t="s">
-        <v>184</v>
+        <v>54</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>185</v>
+        <v>55</v>
       </c>
       <c r="E38" t="s">
-        <v>186</v>
+        <v>56</v>
       </c>
       <c r="F38" s="5">
-        <v>43212</v>
+        <v>40714.365972222222</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>312</v>
+        <v>182</v>
       </c>
       <c r="B39" t="s">
-        <v>313</v>
+        <v>183</v>
       </c>
       <c r="C39" t="s">
-        <v>314</v>
+        <v>184</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>325</v>
+        <v>185</v>
       </c>
       <c r="E39" t="s">
-        <v>315</v>
-      </c>
-      <c r="F39" s="6">
-        <v>44676</v>
+        <v>186</v>
+      </c>
+      <c r="F39" s="5">
+        <v>43212</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>232</v>
+        <v>312</v>
       </c>
       <c r="B40" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="C40" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>220</v>
+        <v>325</v>
       </c>
       <c r="E40" t="s">
-        <v>221</v>
-      </c>
-      <c r="F40" s="5">
-        <v>43973</v>
+        <v>315</v>
+      </c>
+      <c r="F40" s="6">
+        <v>44676</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B41" t="s">
-        <v>223</v>
+        <v>300</v>
       </c>
       <c r="C41" t="s">
-        <v>224</v>
+        <v>301</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="E41" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="F41" s="5">
-        <v>43616</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>34</v>
+        <v>222</v>
       </c>
       <c r="B42" t="s">
-        <v>35</v>
+        <v>223</v>
       </c>
       <c r="C42" t="s">
-        <v>36</v>
+        <v>224</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>37</v>
+        <v>225</v>
       </c>
       <c r="E42" t="s">
-        <v>38</v>
+        <v>226</v>
       </c>
       <c r="F42" s="5">
-        <v>40305.557638888888</v>
+        <v>43616</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>277</v>
+        <v>34</v>
       </c>
       <c r="B43" t="s">
-        <v>278</v>
+        <v>35</v>
       </c>
       <c r="C43" t="s">
-        <v>279</v>
+        <v>36</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>280</v>
+        <v>37</v>
       </c>
       <c r="E43" t="s">
-        <v>281</v>
+        <v>38</v>
       </c>
       <c r="F43" s="5">
-        <v>44580</v>
+        <v>40305.557638888888</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>74</v>
+        <v>277</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>278</v>
       </c>
       <c r="C44" t="s">
-        <v>76</v>
+        <v>279</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>77</v>
+        <v>280</v>
       </c>
       <c r="E44" t="s">
-        <v>78</v>
+        <v>281</v>
       </c>
       <c r="F44" s="5">
-        <v>40966</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>370</v>
+        <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>199</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s">
-        <v>371</v>
+        <v>76</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>372</v>
+        <v>77</v>
       </c>
       <c r="E45" t="s">
-        <v>373</v>
+        <v>78</v>
       </c>
       <c r="F45" s="5">
-        <v>45355</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>374</v>
+        <v>40966</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>316</v>
+        <v>370</v>
       </c>
       <c r="B46" t="s">
-        <v>317</v>
+        <v>199</v>
       </c>
       <c r="C46" t="s">
-        <v>318</v>
+        <v>371</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>319</v>
+        <v>372</v>
       </c>
       <c r="E46" t="s">
-        <v>320</v>
+        <v>373</v>
       </c>
       <c r="F46" s="5">
-        <v>44700</v>
+        <v>45355</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>248</v>
+        <v>316</v>
       </c>
       <c r="B47" t="s">
-        <v>249</v>
+        <v>317</v>
       </c>
       <c r="C47" t="s">
-        <v>250</v>
+        <v>318</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>252</v>
+        <v>319</v>
+      </c>
+      <c r="E47" t="s">
+        <v>320</v>
       </c>
       <c r="F47" s="5">
-        <v>44151</v>
+        <v>44700</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>79</v>
+        <v>248</v>
       </c>
       <c r="B48" t="s">
-        <v>80</v>
+        <v>249</v>
       </c>
       <c r="C48" t="s">
-        <v>81</v>
+        <v>250</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E48" t="s">
-        <v>83</v>
+        <v>251</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>252</v>
       </c>
       <c r="F48" s="5">
-        <v>41736</v>
+        <v>44151</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>219</v>
+        <v>79</v>
       </c>
       <c r="B49" t="s">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="C49" t="s">
-        <v>301</v>
+        <v>81</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>220</v>
+        <v>82</v>
       </c>
       <c r="E49" t="s">
-        <v>221</v>
+        <v>83</v>
       </c>
       <c r="F49" s="5">
-        <v>43614</v>
+        <v>41736</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="B50" t="s">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="C50" t="s">
-        <v>2</v>
+        <v>301</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>3</v>
+        <v>220</v>
       </c>
       <c r="E50" t="s">
-        <v>4</v>
+        <v>221</v>
       </c>
       <c r="F50" s="5">
-        <v>39932.427083333336</v>
+        <v>43614</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E51" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="F51" s="5">
-        <v>40094.793055555558</v>
+        <v>39932.427083333336</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="B52" t="s">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="C52" t="s">
-        <v>96</v>
+        <v>21</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>97</v>
+        <v>22</v>
       </c>
       <c r="E52" t="s">
-        <v>98</v>
+        <v>23</v>
+      </c>
+      <c r="F52" s="5">
+        <v>40094.793055555558</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>381</v>
+        <v>94</v>
       </c>
       <c r="B53" t="s">
-        <v>234</v>
+        <v>95</v>
       </c>
       <c r="C53" t="s">
-        <v>235</v>
+        <v>96</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>384</v>
+        <v>97</v>
       </c>
       <c r="E53" t="s">
-        <v>382</v>
-      </c>
-      <c r="F53" s="5">
-        <v>45419</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>383</v>
+        <v>98</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>436</v>
+        <v>381</v>
       </c>
       <c r="B54" t="s">
-        <v>317</v>
+        <v>234</v>
       </c>
       <c r="C54" t="s">
-        <v>440</v>
+        <v>235</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>437</v>
+        <v>384</v>
       </c>
       <c r="E54" t="s">
-        <v>438</v>
+        <v>382</v>
       </c>
       <c r="F54" s="5">
-        <v>45834</v>
+        <v>45419</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>439</v>
+        <v>383</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>57</v>
+        <v>436</v>
       </c>
       <c r="B55" t="s">
-        <v>58</v>
+        <v>317</v>
       </c>
       <c r="C55" t="s">
-        <v>59</v>
+        <v>440</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>60</v>
+        <v>437</v>
       </c>
       <c r="E55" t="s">
-        <v>61</v>
+        <v>438</v>
       </c>
       <c r="F55" s="5">
-        <v>40854.607638888891</v>
+        <v>45834</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>360</v>
+        <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>361</v>
+        <v>58</v>
       </c>
       <c r="C56" t="s">
-        <v>362</v>
+        <v>59</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>363</v>
+        <v>60</v>
       </c>
       <c r="E56" t="s">
-        <v>214</v>
+        <v>61</v>
       </c>
       <c r="F56" s="5">
-        <v>45147</v>
-      </c>
-      <c r="G56" t="s">
-        <v>364</v>
+        <v>40854.607638888891</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>215</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>75</v>
+        <v>360</v>
+      </c>
+      <c r="B57" t="s">
+        <v>361</v>
       </c>
       <c r="C57" t="s">
-        <v>217</v>
+        <v>362</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>216</v>
+        <v>363</v>
+      </c>
+      <c r="E57" t="s">
+        <v>214</v>
       </c>
       <c r="F57" s="5">
-        <v>43503</v>
+        <v>45147</v>
+      </c>
+      <c r="G57" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>448</v>
-      </c>
-      <c r="B58" t="s">
-        <v>449</v>
+        <v>215</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="C58" t="s">
-        <v>450</v>
+        <v>217</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>451</v>
+        <v>218</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>452</v>
+        <v>216</v>
       </c>
       <c r="F58" s="5">
-        <v>45951</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>453</v>
+        <v>43503</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>62</v>
+        <v>448</v>
       </c>
       <c r="B59" t="s">
-        <v>393</v>
+        <v>449</v>
       </c>
       <c r="C59" t="s">
-        <v>394</v>
+        <v>450</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="E59" t="s">
-        <v>63</v>
-      </c>
-      <c r="F59" s="10" t="s">
-        <v>430</v>
+        <v>451</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="F59" s="5">
+        <v>45951</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>391</v>
+        <v>453</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>115</v>
+        <v>393</v>
       </c>
       <c r="C60" t="s">
-        <v>116</v>
+        <v>394</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>117</v>
+        <v>392</v>
       </c>
       <c r="E60" t="s">
-        <v>118</v>
-      </c>
-      <c r="F60" s="5">
-        <v>41900</v>
+        <v>63</v>
+      </c>
+      <c r="F60" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>428</v>
+        <v>114</v>
       </c>
       <c r="B61" t="s">
-        <v>393</v>
+        <v>115</v>
       </c>
       <c r="C61" t="s">
-        <v>394</v>
+        <v>116</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>392</v>
+        <v>117</v>
       </c>
       <c r="E61" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="F61" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>429</v>
+        <v>41900</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>44</v>
+        <v>428</v>
       </c>
       <c r="B62" t="s">
-        <v>45</v>
+        <v>393</v>
       </c>
       <c r="C62" t="s">
-        <v>46</v>
+        <v>394</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>47</v>
+        <v>392</v>
       </c>
       <c r="E62" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F62" s="5">
-        <v>40560.762499999997</v>
+        <v>45818</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>429</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>365</v>
+        <v>44</v>
       </c>
       <c r="B63" t="s">
-        <v>366</v>
+        <v>45</v>
       </c>
       <c r="C63" t="s">
-        <v>367</v>
+        <v>46</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>368</v>
+        <v>47</v>
       </c>
       <c r="E63" t="s">
-        <v>369</v>
+        <v>48</v>
       </c>
       <c r="F63" s="5">
-        <v>45275</v>
+        <v>40560.762499999997</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>208</v>
+        <v>365</v>
       </c>
       <c r="B64" t="s">
-        <v>209</v>
+        <v>366</v>
       </c>
       <c r="C64" t="s">
-        <v>210</v>
+        <v>367</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>211</v>
+        <v>368</v>
       </c>
       <c r="E64" t="s">
-        <v>212</v>
+        <v>369</v>
       </c>
       <c r="F64" s="5">
-        <v>43502</v>
+        <v>45275</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>282</v>
+        <v>208</v>
       </c>
       <c r="B65" t="s">
-        <v>285</v>
+        <v>209</v>
       </c>
       <c r="C65" t="s">
-        <v>286</v>
+        <v>210</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>287</v>
+        <v>211</v>
       </c>
       <c r="E65" t="s">
-        <v>284</v>
+        <v>212</v>
       </c>
       <c r="F65" s="5">
-        <v>44580</v>
+        <v>43502</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B66" t="s">
         <v>285</v>
@@ -3238,562 +3257,562 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>408</v>
+        <v>283</v>
       </c>
       <c r="B67" t="s">
-        <v>361</v>
+        <v>285</v>
       </c>
       <c r="C67" t="s">
-        <v>362</v>
+        <v>286</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>363</v>
+        <v>287</v>
       </c>
       <c r="E67" t="s">
-        <v>214</v>
+        <v>284</v>
       </c>
       <c r="F67" s="5">
-        <v>45695</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>89</v>
+        <v>408</v>
       </c>
       <c r="B68" t="s">
-        <v>90</v>
+        <v>361</v>
       </c>
       <c r="C68" t="s">
-        <v>91</v>
+        <v>362</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>92</v>
+        <v>363</v>
       </c>
       <c r="E68" t="s">
-        <v>93</v>
+        <v>214</v>
       </c>
       <c r="F68" s="5">
-        <v>41780</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>161</v>
+        <v>89</v>
       </c>
       <c r="B69" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="C69" t="s">
-        <v>163</v>
+        <v>91</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>164</v>
+        <v>92</v>
       </c>
       <c r="E69" t="s">
-        <v>165</v>
+        <v>93</v>
       </c>
       <c r="F69" s="5">
-        <v>42530</v>
+        <v>41780</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>213</v>
+        <v>161</v>
       </c>
       <c r="B70" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="C70" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>122</v>
+        <v>164</v>
       </c>
       <c r="E70" t="s">
-        <v>214</v>
+        <v>165</v>
       </c>
       <c r="F70" s="5">
-        <v>43502</v>
+        <v>42530</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>29</v>
+        <v>213</v>
       </c>
       <c r="B71" t="s">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="C71" t="s">
-        <v>31</v>
+        <v>121</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="E71" t="s">
-        <v>33</v>
+        <v>214</v>
       </c>
       <c r="F71" s="5">
-        <v>40164.4375</v>
+        <v>43502</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>423</v>
+        <v>29</v>
       </c>
       <c r="B72" t="s">
-        <v>424</v>
+        <v>30</v>
       </c>
       <c r="C72" t="s">
-        <v>425</v>
+        <v>31</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>426</v>
+        <v>32</v>
+      </c>
+      <c r="E72" t="s">
+        <v>33</v>
       </c>
       <c r="F72" s="5">
-        <v>45803</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>427</v>
+        <v>40164.4375</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>99</v>
+        <v>423</v>
       </c>
       <c r="B73" t="s">
-        <v>100</v>
+        <v>424</v>
       </c>
       <c r="C73" t="s">
-        <v>101</v>
+        <v>425</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E73" t="s">
-        <v>103</v>
+        <v>426</v>
       </c>
       <c r="F73" s="5">
-        <v>41854</v>
+        <v>45803</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
+        <v>99</v>
+      </c>
+      <c r="B74" t="s">
+        <v>100</v>
+      </c>
+      <c r="C74" t="s">
+        <v>101</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E74" t="s">
+        <v>103</v>
+      </c>
+      <c r="F74" s="5">
+        <v>41854</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
         <v>198</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B75" t="s">
         <v>199</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C75" t="s">
         <v>200</v>
       </c>
-      <c r="D74" s="1" t="s">
+      <c r="D75" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="E74" s="5" t="s">
+      <c r="E75" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="F74" s="6">
+      <c r="F75" s="6">
         <v>37415</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A75" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="B75" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C75" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="E75" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="F75" s="5">
-        <v>43997</v>
-      </c>
-      <c r="G75" s="7" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="7" t="s">
-        <v>460</v>
+        <v>238</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="C76" t="s">
-        <v>462</v>
+        <v>234</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>235</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="E76" t="s">
-        <v>464</v>
+        <v>236</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>237</v>
       </c>
       <c r="F76" s="5">
-        <v>46090</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>465</v>
+        <v>43997</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="C77" t="s">
+        <v>462</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="E77" t="s">
+        <v>464</v>
+      </c>
+      <c r="F77" s="5">
+        <v>46090</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="B77" s="7" t="s">
+      <c r="B78" s="7" t="s">
         <v>455</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="C78" s="7" t="s">
         <v>456</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="D78" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E77" s="7" t="s">
+      <c r="E78" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="F77" s="5">
+      <c r="F78" s="5">
         <v>46038</v>
       </c>
-      <c r="G77" s="1" t="s">
+      <c r="G78" s="1" t="s">
         <v>459</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>253</v>
-      </c>
-      <c r="B78" t="s">
-        <v>254</v>
-      </c>
-      <c r="C78" t="s">
-        <v>255</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E78" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="F78" s="5">
-        <v>44166</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>104</v>
+        <v>253</v>
       </c>
       <c r="B79" t="s">
-        <v>105</v>
+        <v>254</v>
       </c>
       <c r="C79" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E79" t="s">
-        <v>108</v>
+        <v>256</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>257</v>
       </c>
       <c r="F79" s="5">
-        <v>41857</v>
+        <v>44166</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="B80" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="C80" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="E80" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="F80" s="5">
-        <v>42467</v>
+        <v>41857</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B81" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C81" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E81" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="F81" s="5">
-        <v>42420</v>
+        <v>42467</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>227</v>
+        <v>133</v>
       </c>
       <c r="B82" t="s">
-        <v>228</v>
+        <v>134</v>
       </c>
       <c r="C82" t="s">
-        <v>229</v>
+        <v>135</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>230</v>
+        <v>136</v>
       </c>
       <c r="E82" t="s">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="F82" s="5">
-        <v>43973</v>
+        <v>42420</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="B83" t="s">
-        <v>15</v>
+        <v>228</v>
       </c>
       <c r="C83" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="E83" t="s">
-        <v>18</v>
+        <v>231</v>
       </c>
       <c r="F83" s="5">
-        <v>40081.550694444442</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>148</v>
+        <v>14</v>
       </c>
       <c r="B84" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C84" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="E84" t="s">
-        <v>151</v>
+        <v>18</v>
       </c>
       <c r="F84" s="5">
-        <v>42472</v>
+        <v>40081.550694444442</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="B85" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C85" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E85" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="F85" s="5">
-        <v>43054</v>
+        <v>42472</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="B86" t="s">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="C86" t="s">
-        <v>301</v>
+        <v>179</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="E86" t="s">
-        <v>221</v>
+        <v>181</v>
       </c>
       <c r="F86" s="5">
-        <v>43973</v>
+        <v>43054</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="B87" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C87" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>290</v>
+        <v>220</v>
       </c>
       <c r="E87" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="F87" s="5">
-        <v>44580</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>172</v>
+        <v>288</v>
       </c>
       <c r="B88" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
       <c r="C88" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>175</v>
+        <v>290</v>
       </c>
       <c r="E88" t="s">
-        <v>176</v>
+        <v>289</v>
       </c>
       <c r="F88" s="5">
-        <v>42739</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>431</v>
+        <v>172</v>
       </c>
       <c r="B89" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C89" t="s">
-        <v>432</v>
+        <v>174</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>433</v>
+        <v>175</v>
       </c>
       <c r="E89" t="s">
-        <v>434</v>
+        <v>176</v>
       </c>
       <c r="F89" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G89" s="1" t="s">
-        <v>435</v>
+        <v>42739</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>375</v>
+        <v>431</v>
       </c>
       <c r="B90" t="s">
-        <v>376</v>
+        <v>183</v>
       </c>
       <c r="C90" t="s">
-        <v>377</v>
+        <v>432</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="E90" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="F90" s="5">
-        <v>45358</v>
+        <v>45818</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>39</v>
+        <v>375</v>
       </c>
       <c r="B91" t="s">
-        <v>40</v>
+        <v>376</v>
       </c>
       <c r="C91" t="s">
-        <v>41</v>
+        <v>377</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>42</v>
+        <v>378</v>
       </c>
       <c r="E91" t="s">
-        <v>43</v>
+        <v>379</v>
       </c>
       <c r="F91" s="5">
-        <v>40522.519444444442</v>
+        <v>45358</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="B92" t="s">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="C92" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="E92" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="F92" s="5">
-        <v>41890</v>
+        <v>40522.519444444442</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="B93" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="C93" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="E93" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="F93" s="5">
-        <v>42852</v>
+        <v>41890</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>177</v>
+        <v>64</v>
       </c>
       <c r="B94" t="s">
         <v>65</v>
@@ -3813,104 +3832,124 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B95" t="s">
-        <v>204</v>
+        <v>65</v>
       </c>
       <c r="C95" t="s">
-        <v>205</v>
+        <v>66</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="F95" s="6">
-        <v>43487</v>
+        <v>67</v>
+      </c>
+      <c r="E95" t="s">
+        <v>68</v>
+      </c>
+      <c r="F95" s="5">
+        <v>42852</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="B96" t="s">
-        <v>157</v>
+        <v>204</v>
       </c>
       <c r="C96" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E96" t="s">
-        <v>160</v>
-      </c>
-      <c r="F96" s="5">
-        <v>42505</v>
+        <v>206</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F96" s="6">
+        <v>43487</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>409</v>
+        <v>156</v>
       </c>
       <c r="B97" t="s">
-        <v>361</v>
+        <v>157</v>
       </c>
       <c r="C97" t="s">
-        <v>362</v>
+        <v>158</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>363</v>
+        <v>159</v>
       </c>
       <c r="E97" t="s">
-        <v>214</v>
+        <v>160</v>
       </c>
       <c r="F97" s="5">
-        <v>45695</v>
-      </c>
-      <c r="G97" t="s">
-        <v>410</v>
+        <v>42505</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>329</v>
+        <v>409</v>
       </c>
       <c r="B98" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C98" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="E98" t="s">
-        <v>333</v>
+        <v>214</v>
       </c>
       <c r="F98" s="5">
-        <v>44775</v>
+        <v>45695</v>
+      </c>
+      <c r="G98" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
+        <v>329</v>
+      </c>
+      <c r="B99" t="s">
+        <v>330</v>
+      </c>
+      <c r="C99" t="s">
+        <v>331</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E99" t="s">
+        <v>333</v>
+      </c>
+      <c r="F99" s="5">
+        <v>44775</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
         <v>138</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B100" t="s">
         <v>139</v>
       </c>
-      <c r="C99" t="s">
+      <c r="C100" t="s">
         <v>140</v>
       </c>
-      <c r="D99" s="1" t="s">
+      <c r="D100" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E99" t="s">
+      <c r="E100" t="s">
         <v>142</v>
       </c>
-      <c r="F99" s="5">
+      <c r="F100" s="5">
         <v>42439</v>
       </c>
     </row>
@@ -3921,77 +3960,77 @@
     </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="D64" r:id="rId1" xr:uid="{407FC650-7151-6940-B8FA-60477C7D30B1}"/>
-    <hyperlink ref="D70" r:id="rId2" xr:uid="{68E4476D-88C7-5D40-9274-7B03AB299562}"/>
-    <hyperlink ref="D57" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
-    <hyperlink ref="D49" r:id="rId4" xr:uid="{234AD513-3ABE-F545-A037-27824EABDF68}"/>
-    <hyperlink ref="D41" r:id="rId5" xr:uid="{7924D455-5B5F-E641-AB7C-FB4BD03EF051}"/>
-    <hyperlink ref="D82" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
-    <hyperlink ref="D40" r:id="rId7" xr:uid="{7AEF03BC-D893-FF42-BB52-AB9C9480EA0D}"/>
-    <hyperlink ref="D86" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
+    <hyperlink ref="D65" r:id="rId1" xr:uid="{407FC650-7151-6940-B8FA-60477C7D30B1}"/>
+    <hyperlink ref="D71" r:id="rId2" xr:uid="{68E4476D-88C7-5D40-9274-7B03AB299562}"/>
+    <hyperlink ref="D58" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
+    <hyperlink ref="D50" r:id="rId4" xr:uid="{234AD513-3ABE-F545-A037-27824EABDF68}"/>
+    <hyperlink ref="D42" r:id="rId5" xr:uid="{7924D455-5B5F-E641-AB7C-FB4BD03EF051}"/>
+    <hyperlink ref="D83" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
+    <hyperlink ref="D41" r:id="rId7" xr:uid="{7AEF03BC-D893-FF42-BB52-AB9C9480EA0D}"/>
+    <hyperlink ref="D87" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
     <hyperlink ref="D12" r:id="rId9" xr:uid="{D57F2423-845A-9E44-A60D-DEEB1150BE7A}"/>
     <hyperlink ref="D10" r:id="rId10" xr:uid="{0133BED0-2D2B-4A0F-AB7C-D58D8B5F381B}"/>
     <hyperlink ref="D3" r:id="rId11" xr:uid="{5F0875F3-1434-4B08-A87A-2BDF5EEDDAC9}"/>
     <hyperlink ref="D26" r:id="rId12" xr:uid="{61482C13-D6B2-4AFF-AD10-908ABE8BA3F2}"/>
-    <hyperlink ref="D78" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
-    <hyperlink ref="D47" r:id="rId14" xr:uid="{FEB07F00-70C8-4D84-B7DF-B36DF7C6138C}"/>
-    <hyperlink ref="D36" r:id="rId15" xr:uid="{9236AFAC-B489-4804-B65A-1988399CC4C2}"/>
-    <hyperlink ref="D75" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
-    <hyperlink ref="D95" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
-    <hyperlink ref="D74" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
-    <hyperlink ref="D30" r:id="rId19" xr:uid="{178F076F-6CAC-44EB-AA97-31037608AA41}"/>
-    <hyperlink ref="D38" r:id="rId20" xr:uid="{E467E97B-65A6-40E0-A2BA-7875E3A5C2C1}"/>
-    <hyperlink ref="D85" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
-    <hyperlink ref="D94" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
-    <hyperlink ref="D88" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
+    <hyperlink ref="D79" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
+    <hyperlink ref="D48" r:id="rId14" xr:uid="{FEB07F00-70C8-4D84-B7DF-B36DF7C6138C}"/>
+    <hyperlink ref="D37" r:id="rId15" xr:uid="{9236AFAC-B489-4804-B65A-1988399CC4C2}"/>
+    <hyperlink ref="D76" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
+    <hyperlink ref="D96" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
+    <hyperlink ref="D75" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
+    <hyperlink ref="D31" r:id="rId19" xr:uid="{178F076F-6CAC-44EB-AA97-31037608AA41}"/>
+    <hyperlink ref="D39" r:id="rId20" xr:uid="{E467E97B-65A6-40E0-A2BA-7875E3A5C2C1}"/>
+    <hyperlink ref="D86" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
+    <hyperlink ref="D95" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
+    <hyperlink ref="D89" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
     <hyperlink ref="D17" r:id="rId24" xr:uid="{8C069B77-F7A2-4DC6-9D5A-D5138E5E1158}"/>
     <hyperlink ref="D16" r:id="rId25" xr:uid="{C770D7DE-6980-45A2-A8B6-8E4C376C05E3}"/>
-    <hyperlink ref="D69" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
-    <hyperlink ref="D96" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
-    <hyperlink ref="D50" r:id="rId28" xr:uid="{2B927B9E-56D2-4AC7-A24B-BA7FAF44F900}"/>
-    <hyperlink ref="D33" r:id="rId29" xr:uid="{5F9DAD98-7221-4BEC-B311-BF6B1BD6F52E}"/>
-    <hyperlink ref="D83" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
-    <hyperlink ref="D51" r:id="rId31" xr:uid="{7BC6DF64-9FBB-461B-BEE3-D705D5A5711D}"/>
+    <hyperlink ref="D70" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
+    <hyperlink ref="D97" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
+    <hyperlink ref="D51" r:id="rId28" xr:uid="{2B927B9E-56D2-4AC7-A24B-BA7FAF44F900}"/>
+    <hyperlink ref="D34" r:id="rId29" xr:uid="{5F9DAD98-7221-4BEC-B311-BF6B1BD6F52E}"/>
+    <hyperlink ref="D84" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
+    <hyperlink ref="D52" r:id="rId31" xr:uid="{7BC6DF64-9FBB-461B-BEE3-D705D5A5711D}"/>
     <hyperlink ref="D21" r:id="rId32" xr:uid="{EE5546A8-9D18-43D6-949A-451AA8A97E76}"/>
-    <hyperlink ref="D71" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
-    <hyperlink ref="D42" r:id="rId34" xr:uid="{03938AC4-898D-4B60-9A83-CF770912371F}"/>
-    <hyperlink ref="D91" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
-    <hyperlink ref="D62" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
+    <hyperlink ref="D72" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
+    <hyperlink ref="D43" r:id="rId34" xr:uid="{03938AC4-898D-4B60-9A83-CF770912371F}"/>
+    <hyperlink ref="D92" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
+    <hyperlink ref="D63" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
     <hyperlink ref="D7" r:id="rId37" xr:uid="{C501338A-FD0F-4F45-B8B1-BD737635609F}"/>
-    <hyperlink ref="D37" r:id="rId38" xr:uid="{973F790E-4686-49DC-8382-D85663F42FE4}"/>
-    <hyperlink ref="D55" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
-    <hyperlink ref="D93" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
+    <hyperlink ref="D38" r:id="rId38" xr:uid="{973F790E-4686-49DC-8382-D85663F42FE4}"/>
+    <hyperlink ref="D56" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
+    <hyperlink ref="D94" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
     <hyperlink ref="D13" r:id="rId41" xr:uid="{E0321D7C-4A33-425C-AC81-F2844EF49280}"/>
-    <hyperlink ref="D44" r:id="rId42" xr:uid="{9362C2F6-92F8-4578-90F4-F93A12DB0620}"/>
-    <hyperlink ref="D48" r:id="rId43" xr:uid="{3D2507DB-58F1-46EB-972C-7262C11F3BC0}"/>
+    <hyperlink ref="D45" r:id="rId42" xr:uid="{9362C2F6-92F8-4578-90F4-F93A12DB0620}"/>
+    <hyperlink ref="D49" r:id="rId43" xr:uid="{3D2507DB-58F1-46EB-972C-7262C11F3BC0}"/>
     <hyperlink ref="D15" r:id="rId44" xr:uid="{FD7129AB-69C9-448B-90D0-0EB16503D948}"/>
-    <hyperlink ref="D68" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
-    <hyperlink ref="D52" r:id="rId46" xr:uid="{FA35DE19-FE12-4948-8782-601512787A1F}"/>
-    <hyperlink ref="D73" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
-    <hyperlink ref="D79" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
-    <hyperlink ref="D92" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
-    <hyperlink ref="D60" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
+    <hyperlink ref="D69" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
+    <hyperlink ref="D53" r:id="rId46" xr:uid="{FA35DE19-FE12-4948-8782-601512787A1F}"/>
+    <hyperlink ref="D74" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
+    <hyperlink ref="D80" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
+    <hyperlink ref="D93" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
+    <hyperlink ref="D61" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
     <hyperlink ref="D27" r:id="rId51" xr:uid="{20CCBF4F-DA07-40B1-84D7-9C64B10A18DD}"/>
     <hyperlink ref="D4" r:id="rId52" xr:uid="{04F40983-3CCF-4A98-9D71-83239E621071}"/>
-    <hyperlink ref="D32" r:id="rId53" xr:uid="{B6182D1F-82B7-4DC3-BB62-5D4CE3E6347D}"/>
-    <hyperlink ref="D81" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
-    <hyperlink ref="D99" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
-    <hyperlink ref="D80" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
-    <hyperlink ref="D84" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
+    <hyperlink ref="D33" r:id="rId53" xr:uid="{B6182D1F-82B7-4DC3-BB62-5D4CE3E6347D}"/>
+    <hyperlink ref="D82" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
+    <hyperlink ref="D100" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
+    <hyperlink ref="D81" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
+    <hyperlink ref="D85" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
     <hyperlink ref="D9" r:id="rId58" xr:uid="{F7E14BE7-9BEF-429A-BC06-CA914EDCD03E}"/>
     <hyperlink ref="D23" r:id="rId59" xr:uid="{13F0A7EA-4265-4C1A-936D-0F1F22648B66}"/>
-    <hyperlink ref="D43" r:id="rId60" display="mailto:david@zwang.com" xr:uid="{2E031ABA-CF1B-48A8-96E6-B6DCE94345AE}"/>
-    <hyperlink ref="D65" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
-    <hyperlink ref="D66" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
-    <hyperlink ref="D87" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
-    <hyperlink ref="D29" r:id="rId64" xr:uid="{3AD048BB-9D70-41FA-8645-47CF1BE084C9}"/>
-    <hyperlink ref="D31" r:id="rId65" display="mailto:bertvk@enfocus.com" xr:uid="{6F56AFA2-CA54-4A51-B51B-36740F243F7A}"/>
-    <hyperlink ref="D46" r:id="rId66" xr:uid="{DEECD580-BF33-4FBB-A267-48E6674FF044}"/>
-    <hyperlink ref="D34" r:id="rId67" xr:uid="{3A6EE0DA-E93B-4D24-AD52-FF9D72BBC152}"/>
+    <hyperlink ref="D44" r:id="rId60" display="mailto:david@zwang.com" xr:uid="{2E031ABA-CF1B-48A8-96E6-B6DCE94345AE}"/>
+    <hyperlink ref="D66" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
+    <hyperlink ref="D67" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
+    <hyperlink ref="D88" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
+    <hyperlink ref="D30" r:id="rId64" xr:uid="{3AD048BB-9D70-41FA-8645-47CF1BE084C9}"/>
+    <hyperlink ref="D32" r:id="rId65" display="mailto:bertvk@enfocus.com" xr:uid="{6F56AFA2-CA54-4A51-B51B-36740F243F7A}"/>
+    <hyperlink ref="D47" r:id="rId66" xr:uid="{DEECD580-BF33-4FBB-A267-48E6674FF044}"/>
+    <hyperlink ref="D35" r:id="rId67" xr:uid="{3A6EE0DA-E93B-4D24-AD52-FF9D72BBC152}"/>
     <hyperlink ref="D19" r:id="rId68" xr:uid="{897A4DB8-756C-42E5-AF7B-011BBBE00628}"/>
-    <hyperlink ref="D39" r:id="rId69" xr:uid="{47A4E692-159B-4E48-A1D4-411E278B3A43}"/>
+    <hyperlink ref="D40" r:id="rId69" xr:uid="{47A4E692-159B-4E48-A1D4-411E278B3A43}"/>
     <hyperlink ref="D2" r:id="rId70" display="mailto:frank.vyncke@yin4yang.com" xr:uid="{E29600CB-349C-4C55-AC29-3B61912C4757}"/>
-    <hyperlink ref="D98" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
+    <hyperlink ref="D99" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
     <hyperlink ref="D25" r:id="rId72" xr:uid="{BF5FD244-0DE0-493E-A7E1-0CEDCE9B77AA}"/>
     <hyperlink ref="D5" r:id="rId73" xr:uid="{33D12C26-CC5E-4925-86B6-4AE855A6371F}"/>
     <hyperlink ref="G5" r:id="rId74" xr:uid="{2FA39695-7884-42EC-9380-C8EFD7B7EAD9}"/>
@@ -4000,45 +4039,46 @@
     <hyperlink ref="G6" r:id="rId77" xr:uid="{EF6627CA-3B1A-440B-85D4-A1B7067549BD}"/>
     <hyperlink ref="D11" r:id="rId78" xr:uid="{058D1BE7-4CFF-4740-BC92-2074C717A677}"/>
     <hyperlink ref="G11" r:id="rId79" xr:uid="{B9062A46-48F6-45FB-8197-4FD986CC482D}"/>
-    <hyperlink ref="D56" r:id="rId80" xr:uid="{0CFEC845-7F90-4802-9D24-4AC8905CD11B}"/>
-    <hyperlink ref="D63" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
-    <hyperlink ref="D45" r:id="rId82" xr:uid="{72B2BA10-0B55-4ACF-9CC1-DA30FB4C2741}"/>
-    <hyperlink ref="G45" r:id="rId83" xr:uid="{1106BFBB-F6F3-4E8A-8B65-06381130271C}"/>
-    <hyperlink ref="D90" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
-    <hyperlink ref="G90" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
-    <hyperlink ref="G53" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
-    <hyperlink ref="D53" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
+    <hyperlink ref="D57" r:id="rId80" xr:uid="{0CFEC845-7F90-4802-9D24-4AC8905CD11B}"/>
+    <hyperlink ref="D64" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
+    <hyperlink ref="D46" r:id="rId82" xr:uid="{72B2BA10-0B55-4ACF-9CC1-DA30FB4C2741}"/>
+    <hyperlink ref="G46" r:id="rId83" xr:uid="{1106BFBB-F6F3-4E8A-8B65-06381130271C}"/>
+    <hyperlink ref="D91" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
+    <hyperlink ref="G91" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
+    <hyperlink ref="G54" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
+    <hyperlink ref="D54" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
     <hyperlink ref="G20" r:id="rId88" xr:uid="{C64F139E-8286-4E7A-8B5E-9D69FC9A0C25}"/>
-    <hyperlink ref="G59" r:id="rId89" xr:uid="{5D505EE9-2263-469C-9455-D353F4C9921E}"/>
-    <hyperlink ref="D59" r:id="rId90" xr:uid="{5715AC7F-4208-4141-884D-FD2EB9CB5E95}"/>
+    <hyperlink ref="G60" r:id="rId89" xr:uid="{5D505EE9-2263-469C-9455-D353F4C9921E}"/>
+    <hyperlink ref="D60" r:id="rId90" xr:uid="{5715AC7F-4208-4141-884D-FD2EB9CB5E95}"/>
     <hyperlink ref="D18" r:id="rId91" xr:uid="{50E71DF8-A245-41B4-83A8-E6488454D9A4}"/>
     <hyperlink ref="G28" r:id="rId92" xr:uid="{15520162-C027-42E1-8EC1-CA7EA9FD18BC}"/>
     <hyperlink ref="D28" r:id="rId93" xr:uid="{E9A12839-D069-4292-A5EA-36394565B8A0}"/>
-    <hyperlink ref="D35" r:id="rId94" xr:uid="{F07464A9-7B4E-4E5B-9EEE-3F687E9DC9AC}"/>
-    <hyperlink ref="G35" r:id="rId95" xr:uid="{73C68A69-730D-4676-B564-01BC2FDA7E73}"/>
-    <hyperlink ref="D67" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
-    <hyperlink ref="D97" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
+    <hyperlink ref="D36" r:id="rId94" xr:uid="{F07464A9-7B4E-4E5B-9EEE-3F687E9DC9AC}"/>
+    <hyperlink ref="G36" r:id="rId95" xr:uid="{73C68A69-730D-4676-B564-01BC2FDA7E73}"/>
+    <hyperlink ref="D68" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
+    <hyperlink ref="D98" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
     <hyperlink ref="D22" r:id="rId98" xr:uid="{3C768ED5-B6E7-416A-B3CF-31E9B14F1258}"/>
     <hyperlink ref="G22" r:id="rId99" xr:uid="{5C4AC9BE-92AA-40F8-AA34-D54E19486DEE}"/>
     <hyperlink ref="D8" r:id="rId100" xr:uid="{0DDFD3D5-41E0-4A59-8992-A1EE6FD3C05D}"/>
     <hyperlink ref="G8" r:id="rId101" xr:uid="{82F38FA1-9E55-4CDE-87F7-9C87D20D9E51}"/>
-    <hyperlink ref="D72" r:id="rId102" xr:uid="{F47445AD-9EE1-46DB-B7BA-B288E5B3A5E1}"/>
-    <hyperlink ref="G72" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
-    <hyperlink ref="G61" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
-    <hyperlink ref="D61" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
-    <hyperlink ref="D89" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
-    <hyperlink ref="G89" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
-    <hyperlink ref="D54" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
-    <hyperlink ref="G54" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
+    <hyperlink ref="D73" r:id="rId102" xr:uid="{F47445AD-9EE1-46DB-B7BA-B288E5B3A5E1}"/>
+    <hyperlink ref="G73" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
+    <hyperlink ref="G62" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
+    <hyperlink ref="D62" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
+    <hyperlink ref="D90" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
+    <hyperlink ref="G90" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
+    <hyperlink ref="D55" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
+    <hyperlink ref="G55" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
     <hyperlink ref="D24" r:id="rId110" xr:uid="{42EF2DCB-F6A9-4EC5-9C1C-9B9A137FDD6C}"/>
     <hyperlink ref="G24" r:id="rId111" xr:uid="{68016CF6-F4CA-4852-AF56-7954DB739663}"/>
-    <hyperlink ref="D58" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
-    <hyperlink ref="G58" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
-    <hyperlink ref="D77" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
-    <hyperlink ref="G77" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
-    <hyperlink ref="G76" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
+    <hyperlink ref="D59" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
+    <hyperlink ref="G59" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
+    <hyperlink ref="D78" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
+    <hyperlink ref="G78" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
+    <hyperlink ref="G77" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
+    <hyperlink ref="D29" r:id="rId117" xr:uid="{B822E1EC-0934-422A-B4A5-1DB34262685E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId117"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId118"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve #56 for LGEN
</commit_message>
<xml_diff>
--- a/ISO PDF Registry.xlsx
+++ b/ISO PDF Registry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\share\pdf-names-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6AD0B4F-243B-4026-9F32-22E88E153248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DFFA40-C60F-4E1F-B436-4EC649609E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="4920" windowWidth="21600" windowHeight="13560" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
+    <workbookView xWindow="3456" yWindow="3456" windowWidth="21600" windowHeight="13560" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
   </bookViews>
   <sheets>
     <sheet name="PDF Prefix Registry" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="478">
   <si>
     <t>ITXT</t>
   </si>
@@ -1446,6 +1446,24 @@
   </si>
   <si>
     <t>"PDFA" cannot be used</t>
+  </si>
+  <si>
+    <t>LGEN</t>
+  </si>
+  <si>
+    <t>Christian</t>
+  </si>
+  <si>
+    <t>Nyffenegger</t>
+  </si>
+  <si>
+    <t>Link Genetic GmbH</t>
+  </si>
+  <si>
+    <t>https://github.com/adobe/pdf-names-list/issues/56</t>
+  </si>
+  <si>
+    <t>Christian.Nyffenegger@linkgenetic.com</t>
   </si>
 </sst>
 </file>
@@ -1869,7 +1887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E74889-C943-2949-BDAA-069F646F779D}">
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
@@ -2988,285 +3006,288 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>381</v>
+        <v>472</v>
       </c>
       <c r="B54" t="s">
-        <v>234</v>
+        <v>473</v>
       </c>
       <c r="C54" t="s">
-        <v>235</v>
+        <v>474</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>384</v>
+        <v>477</v>
       </c>
       <c r="E54" t="s">
-        <v>382</v>
+        <v>475</v>
       </c>
       <c r="F54" s="5">
-        <v>45419</v>
+        <v>46155</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>383</v>
+        <v>476</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>436</v>
+        <v>381</v>
       </c>
       <c r="B55" t="s">
-        <v>317</v>
+        <v>234</v>
       </c>
       <c r="C55" t="s">
-        <v>440</v>
+        <v>235</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>437</v>
+        <v>384</v>
       </c>
       <c r="E55" t="s">
-        <v>438</v>
+        <v>382</v>
       </c>
       <c r="F55" s="5">
-        <v>45834</v>
+        <v>45419</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>439</v>
+        <v>383</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>436</v>
       </c>
       <c r="B56" t="s">
-        <v>58</v>
+        <v>317</v>
       </c>
       <c r="C56" t="s">
-        <v>59</v>
+        <v>440</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>60</v>
+        <v>437</v>
       </c>
       <c r="E56" t="s">
-        <v>61</v>
+        <v>438</v>
       </c>
       <c r="F56" s="5">
-        <v>40854.607638888891</v>
+        <v>45834</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>360</v>
+        <v>57</v>
       </c>
       <c r="B57" t="s">
-        <v>361</v>
+        <v>58</v>
       </c>
       <c r="C57" t="s">
-        <v>362</v>
+        <v>59</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>363</v>
+        <v>60</v>
       </c>
       <c r="E57" t="s">
-        <v>214</v>
+        <v>61</v>
       </c>
       <c r="F57" s="5">
-        <v>45147</v>
-      </c>
-      <c r="G57" t="s">
-        <v>364</v>
+        <v>40854.607638888891</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>215</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>75</v>
+        <v>360</v>
+      </c>
+      <c r="B58" t="s">
+        <v>361</v>
       </c>
       <c r="C58" t="s">
-        <v>217</v>
+        <v>362</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>216</v>
+        <v>363</v>
+      </c>
+      <c r="E58" t="s">
+        <v>214</v>
       </c>
       <c r="F58" s="5">
-        <v>43503</v>
+        <v>45147</v>
+      </c>
+      <c r="G58" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>448</v>
-      </c>
-      <c r="B59" t="s">
-        <v>449</v>
+        <v>215</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="C59" t="s">
-        <v>450</v>
+        <v>217</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>451</v>
+        <v>218</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>452</v>
+        <v>216</v>
       </c>
       <c r="F59" s="5">
-        <v>45951</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>453</v>
+        <v>43503</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>62</v>
+        <v>448</v>
       </c>
       <c r="B60" t="s">
-        <v>393</v>
+        <v>449</v>
       </c>
       <c r="C60" t="s">
-        <v>394</v>
+        <v>450</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="E60" t="s">
-        <v>63</v>
-      </c>
-      <c r="F60" s="10" t="s">
-        <v>430</v>
+        <v>451</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="F60" s="5">
+        <v>45951</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>391</v>
+        <v>453</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>115</v>
+        <v>393</v>
       </c>
       <c r="C61" t="s">
-        <v>116</v>
+        <v>394</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>117</v>
+        <v>392</v>
       </c>
       <c r="E61" t="s">
-        <v>118</v>
-      </c>
-      <c r="F61" s="5">
-        <v>41900</v>
+        <v>63</v>
+      </c>
+      <c r="F61" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>428</v>
+        <v>114</v>
       </c>
       <c r="B62" t="s">
-        <v>393</v>
+        <v>115</v>
       </c>
       <c r="C62" t="s">
-        <v>394</v>
+        <v>116</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>392</v>
+        <v>117</v>
       </c>
       <c r="E62" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="F62" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>429</v>
+        <v>41900</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>44</v>
+        <v>428</v>
       </c>
       <c r="B63" t="s">
-        <v>45</v>
+        <v>393</v>
       </c>
       <c r="C63" t="s">
-        <v>46</v>
+        <v>394</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>47</v>
+        <v>392</v>
       </c>
       <c r="E63" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F63" s="5">
-        <v>40560.762499999997</v>
+        <v>45818</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>429</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>365</v>
+        <v>44</v>
       </c>
       <c r="B64" t="s">
-        <v>366</v>
+        <v>45</v>
       </c>
       <c r="C64" t="s">
-        <v>367</v>
+        <v>46</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>368</v>
+        <v>47</v>
       </c>
       <c r="E64" t="s">
-        <v>369</v>
+        <v>48</v>
       </c>
       <c r="F64" s="5">
-        <v>45275</v>
+        <v>40560.762499999997</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>208</v>
+        <v>365</v>
       </c>
       <c r="B65" t="s">
-        <v>209</v>
+        <v>366</v>
       </c>
       <c r="C65" t="s">
-        <v>210</v>
+        <v>367</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>211</v>
+        <v>368</v>
       </c>
       <c r="E65" t="s">
-        <v>212</v>
+        <v>369</v>
       </c>
       <c r="F65" s="5">
-        <v>43502</v>
+        <v>45275</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>282</v>
+        <v>208</v>
       </c>
       <c r="B66" t="s">
-        <v>285</v>
+        <v>209</v>
       </c>
       <c r="C66" t="s">
-        <v>286</v>
+        <v>210</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>287</v>
+        <v>211</v>
       </c>
       <c r="E66" t="s">
-        <v>284</v>
+        <v>212</v>
       </c>
       <c r="F66" s="5">
-        <v>44580</v>
+        <v>43502</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B67" t="s">
         <v>285</v>
@@ -3286,90 +3307,87 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>408</v>
+        <v>283</v>
       </c>
       <c r="B68" t="s">
-        <v>361</v>
+        <v>285</v>
       </c>
       <c r="C68" t="s">
-        <v>362</v>
+        <v>286</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>363</v>
+        <v>287</v>
       </c>
       <c r="E68" t="s">
-        <v>214</v>
+        <v>284</v>
       </c>
       <c r="F68" s="5">
-        <v>45695</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>89</v>
+        <v>408</v>
       </c>
       <c r="B69" t="s">
-        <v>90</v>
+        <v>361</v>
       </c>
       <c r="C69" t="s">
-        <v>91</v>
+        <v>362</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>92</v>
+        <v>363</v>
       </c>
       <c r="E69" t="s">
-        <v>93</v>
+        <v>214</v>
       </c>
       <c r="F69" s="5">
-        <v>41780</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>161</v>
+        <v>89</v>
       </c>
       <c r="B70" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>163</v>
+        <v>91</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>164</v>
+        <v>92</v>
       </c>
       <c r="E70" t="s">
-        <v>165</v>
+        <v>93</v>
       </c>
       <c r="F70" s="5">
-        <v>42530</v>
+        <v>41780</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>469</v>
+        <v>161</v>
       </c>
       <c r="B71" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="C71" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>122</v>
+        <v>164</v>
       </c>
       <c r="E71" t="s">
-        <v>214</v>
+        <v>165</v>
       </c>
       <c r="F71" s="5">
-        <v>46147</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>470</v>
+        <v>42530</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>213</v>
+        <v>469</v>
       </c>
       <c r="B72" t="s">
         <v>120</v>
@@ -3384,490 +3402,493 @@
         <v>214</v>
       </c>
       <c r="F72" s="5">
-        <v>43502</v>
-      </c>
-      <c r="G72" t="s">
-        <v>471</v>
+        <v>46147</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>29</v>
+        <v>213</v>
       </c>
       <c r="B73" t="s">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="C73" t="s">
-        <v>31</v>
+        <v>121</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="E73" t="s">
-        <v>33</v>
+        <v>214</v>
       </c>
       <c r="F73" s="5">
-        <v>40164.4375</v>
+        <v>43502</v>
+      </c>
+      <c r="G73" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>423</v>
+        <v>29</v>
       </c>
       <c r="B74" t="s">
-        <v>424</v>
+        <v>30</v>
       </c>
       <c r="C74" t="s">
-        <v>425</v>
+        <v>31</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>426</v>
+        <v>32</v>
+      </c>
+      <c r="E74" t="s">
+        <v>33</v>
       </c>
       <c r="F74" s="5">
-        <v>45803</v>
-      </c>
-      <c r="G74" s="1" t="s">
-        <v>427</v>
+        <v>40164.4375</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>99</v>
+        <v>423</v>
       </c>
       <c r="B75" t="s">
-        <v>100</v>
+        <v>424</v>
       </c>
       <c r="C75" t="s">
-        <v>101</v>
+        <v>425</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E75" t="s">
-        <v>103</v>
+        <v>426</v>
       </c>
       <c r="F75" s="5">
-        <v>41854</v>
+        <v>45803</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
+        <v>99</v>
+      </c>
+      <c r="B76" t="s">
+        <v>100</v>
+      </c>
+      <c r="C76" t="s">
+        <v>101</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E76" t="s">
+        <v>103</v>
+      </c>
+      <c r="F76" s="5">
+        <v>41854</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
         <v>198</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B77" t="s">
         <v>199</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C77" t="s">
         <v>200</v>
       </c>
-      <c r="D76" s="1" t="s">
+      <c r="D77" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="E76" s="5" t="s">
+      <c r="E77" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="F76" s="6">
+      <c r="F77" s="6">
         <v>37415</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A77" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C77" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="F77" s="5">
-        <v>43997</v>
-      </c>
-      <c r="G77" s="7" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="7" t="s">
-        <v>460</v>
+        <v>238</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="C78" t="s">
-        <v>462</v>
+        <v>234</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>235</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="E78" t="s">
-        <v>464</v>
+        <v>236</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>237</v>
       </c>
       <c r="F78" s="5">
-        <v>46090</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>465</v>
+        <v>43997</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="C79" t="s">
+        <v>462</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="E79" t="s">
+        <v>464</v>
+      </c>
+      <c r="F79" s="5">
+        <v>46090</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="B79" s="7" t="s">
+      <c r="B80" s="7" t="s">
         <v>455</v>
       </c>
-      <c r="C79" s="7" t="s">
+      <c r="C80" s="7" t="s">
         <v>456</v>
       </c>
-      <c r="D79" s="1" t="s">
+      <c r="D80" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E79" s="7" t="s">
+      <c r="E80" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="F79" s="5">
+      <c r="F80" s="5">
         <v>46038</v>
       </c>
-      <c r="G79" s="1" t="s">
+      <c r="G80" s="1" t="s">
         <v>459</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>253</v>
-      </c>
-      <c r="B80" t="s">
-        <v>254</v>
-      </c>
-      <c r="C80" t="s">
-        <v>255</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E80" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="F80" s="5">
-        <v>44166</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>104</v>
+        <v>253</v>
       </c>
       <c r="B81" t="s">
-        <v>105</v>
+        <v>254</v>
       </c>
       <c r="C81" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E81" t="s">
-        <v>108</v>
+        <v>256</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>257</v>
       </c>
       <c r="F81" s="5">
-        <v>41857</v>
+        <v>44166</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="B82" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="C82" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="E82" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="F82" s="5">
-        <v>42467</v>
+        <v>41857</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B83" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C83" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E83" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="F83" s="5">
-        <v>42420</v>
+        <v>42467</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>227</v>
+        <v>133</v>
       </c>
       <c r="B84" t="s">
-        <v>228</v>
+        <v>134</v>
       </c>
       <c r="C84" t="s">
-        <v>229</v>
+        <v>135</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>230</v>
+        <v>136</v>
       </c>
       <c r="E84" t="s">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="F84" s="5">
-        <v>43973</v>
+        <v>42420</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="B85" t="s">
-        <v>15</v>
+        <v>228</v>
       </c>
       <c r="C85" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="E85" t="s">
-        <v>18</v>
+        <v>231</v>
       </c>
       <c r="F85" s="5">
-        <v>40081.550694444442</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>148</v>
+        <v>14</v>
       </c>
       <c r="B86" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C86" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="E86" t="s">
-        <v>151</v>
+        <v>18</v>
       </c>
       <c r="F86" s="5">
-        <v>42472</v>
+        <v>40081.550694444442</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="B87" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C87" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E87" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="F87" s="5">
-        <v>43054</v>
+        <v>42472</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="B88" t="s">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="C88" t="s">
-        <v>301</v>
+        <v>179</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="E88" t="s">
-        <v>221</v>
+        <v>181</v>
       </c>
       <c r="F88" s="5">
-        <v>43973</v>
+        <v>43054</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="B89" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C89" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>290</v>
+        <v>220</v>
       </c>
       <c r="E89" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="F89" s="5">
-        <v>44580</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>172</v>
+        <v>288</v>
       </c>
       <c r="B90" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
       <c r="C90" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>175</v>
+        <v>290</v>
       </c>
       <c r="E90" t="s">
-        <v>176</v>
+        <v>289</v>
       </c>
       <c r="F90" s="5">
-        <v>42739</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>431</v>
+        <v>172</v>
       </c>
       <c r="B91" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C91" t="s">
-        <v>432</v>
+        <v>174</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>433</v>
+        <v>175</v>
       </c>
       <c r="E91" t="s">
-        <v>434</v>
+        <v>176</v>
       </c>
       <c r="F91" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G91" s="1" t="s">
-        <v>435</v>
+        <v>42739</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>375</v>
+        <v>431</v>
       </c>
       <c r="B92" t="s">
-        <v>376</v>
+        <v>183</v>
       </c>
       <c r="C92" t="s">
-        <v>377</v>
+        <v>432</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="E92" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="F92" s="5">
-        <v>45358</v>
+        <v>45818</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>39</v>
+        <v>375</v>
       </c>
       <c r="B93" t="s">
-        <v>40</v>
+        <v>376</v>
       </c>
       <c r="C93" t="s">
-        <v>41</v>
+        <v>377</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>42</v>
+        <v>378</v>
       </c>
       <c r="E93" t="s">
-        <v>43</v>
+        <v>379</v>
       </c>
       <c r="F93" s="5">
-        <v>40522.519444444442</v>
+        <v>45358</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="B94" t="s">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="C94" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="E94" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="F94" s="5">
-        <v>41890</v>
+        <v>40522.519444444442</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="B95" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="C95" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="E95" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="F95" s="5">
-        <v>42852</v>
+        <v>41890</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>177</v>
+        <v>64</v>
       </c>
       <c r="B96" t="s">
         <v>65</v>
@@ -3887,104 +3908,124 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B97" t="s">
-        <v>204</v>
+        <v>65</v>
       </c>
       <c r="C97" t="s">
-        <v>205</v>
+        <v>66</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="F97" s="6">
-        <v>43487</v>
+        <v>67</v>
+      </c>
+      <c r="E97" t="s">
+        <v>68</v>
+      </c>
+      <c r="F97" s="5">
+        <v>42852</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="B98" t="s">
-        <v>157</v>
+        <v>204</v>
       </c>
       <c r="C98" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E98" t="s">
-        <v>160</v>
-      </c>
-      <c r="F98" s="5">
-        <v>42505</v>
+        <v>206</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F98" s="6">
+        <v>43487</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>409</v>
+        <v>156</v>
       </c>
       <c r="B99" t="s">
-        <v>361</v>
+        <v>157</v>
       </c>
       <c r="C99" t="s">
-        <v>362</v>
+        <v>158</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>363</v>
+        <v>159</v>
       </c>
       <c r="E99" t="s">
-        <v>214</v>
+        <v>160</v>
       </c>
       <c r="F99" s="5">
-        <v>45695</v>
-      </c>
-      <c r="G99" t="s">
-        <v>410</v>
+        <v>42505</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>329</v>
+        <v>409</v>
       </c>
       <c r="B100" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C100" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="E100" t="s">
-        <v>333</v>
+        <v>214</v>
       </c>
       <c r="F100" s="5">
-        <v>44775</v>
+        <v>45695</v>
+      </c>
+      <c r="G100" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
+        <v>329</v>
+      </c>
+      <c r="B101" t="s">
+        <v>330</v>
+      </c>
+      <c r="C101" t="s">
+        <v>331</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E101" t="s">
+        <v>333</v>
+      </c>
+      <c r="F101" s="5">
+        <v>44775</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
         <v>138</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B102" t="s">
         <v>139</v>
       </c>
-      <c r="C101" t="s">
+      <c r="C102" t="s">
         <v>140</v>
       </c>
-      <c r="D101" s="1" t="s">
+      <c r="D102" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E101" t="s">
+      <c r="E102" t="s">
         <v>142</v>
       </c>
-      <c r="F101" s="5">
+      <c r="F102" s="5">
         <v>42439</v>
       </c>
     </row>
@@ -3995,69 +4036,69 @@
     </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="D65" r:id="rId1" xr:uid="{407FC650-7151-6940-B8FA-60477C7D30B1}"/>
-    <hyperlink ref="D72" r:id="rId2" xr:uid="{68E4476D-88C7-5D40-9274-7B03AB299562}"/>
-    <hyperlink ref="D58" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
+    <hyperlink ref="D66" r:id="rId1" xr:uid="{407FC650-7151-6940-B8FA-60477C7D30B1}"/>
+    <hyperlink ref="D73" r:id="rId2" xr:uid="{68E4476D-88C7-5D40-9274-7B03AB299562}"/>
+    <hyperlink ref="D59" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
     <hyperlink ref="D50" r:id="rId4" xr:uid="{234AD513-3ABE-F545-A037-27824EABDF68}"/>
     <hyperlink ref="D42" r:id="rId5" xr:uid="{7924D455-5B5F-E641-AB7C-FB4BD03EF051}"/>
-    <hyperlink ref="D84" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
+    <hyperlink ref="D85" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
     <hyperlink ref="D41" r:id="rId7" xr:uid="{7AEF03BC-D893-FF42-BB52-AB9C9480EA0D}"/>
-    <hyperlink ref="D88" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
+    <hyperlink ref="D89" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
     <hyperlink ref="D12" r:id="rId9" xr:uid="{D57F2423-845A-9E44-A60D-DEEB1150BE7A}"/>
     <hyperlink ref="D10" r:id="rId10" xr:uid="{0133BED0-2D2B-4A0F-AB7C-D58D8B5F381B}"/>
     <hyperlink ref="D3" r:id="rId11" xr:uid="{5F0875F3-1434-4B08-A87A-2BDF5EEDDAC9}"/>
     <hyperlink ref="D26" r:id="rId12" xr:uid="{61482C13-D6B2-4AFF-AD10-908ABE8BA3F2}"/>
-    <hyperlink ref="D80" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
+    <hyperlink ref="D81" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
     <hyperlink ref="D48" r:id="rId14" xr:uid="{FEB07F00-70C8-4D84-B7DF-B36DF7C6138C}"/>
     <hyperlink ref="D37" r:id="rId15" xr:uid="{9236AFAC-B489-4804-B65A-1988399CC4C2}"/>
-    <hyperlink ref="D77" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
-    <hyperlink ref="D97" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
-    <hyperlink ref="D76" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
+    <hyperlink ref="D78" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
+    <hyperlink ref="D98" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
+    <hyperlink ref="D77" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
     <hyperlink ref="D31" r:id="rId19" xr:uid="{178F076F-6CAC-44EB-AA97-31037608AA41}"/>
     <hyperlink ref="D39" r:id="rId20" xr:uid="{E467E97B-65A6-40E0-A2BA-7875E3A5C2C1}"/>
-    <hyperlink ref="D87" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
-    <hyperlink ref="D96" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
-    <hyperlink ref="D90" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
+    <hyperlink ref="D88" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
+    <hyperlink ref="D97" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
+    <hyperlink ref="D91" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
     <hyperlink ref="D17" r:id="rId24" xr:uid="{8C069B77-F7A2-4DC6-9D5A-D5138E5E1158}"/>
     <hyperlink ref="D16" r:id="rId25" xr:uid="{C770D7DE-6980-45A2-A8B6-8E4C376C05E3}"/>
-    <hyperlink ref="D70" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
-    <hyperlink ref="D98" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
+    <hyperlink ref="D71" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
+    <hyperlink ref="D99" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
     <hyperlink ref="D51" r:id="rId28" xr:uid="{2B927B9E-56D2-4AC7-A24B-BA7FAF44F900}"/>
     <hyperlink ref="D34" r:id="rId29" xr:uid="{5F9DAD98-7221-4BEC-B311-BF6B1BD6F52E}"/>
-    <hyperlink ref="D85" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
+    <hyperlink ref="D86" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
     <hyperlink ref="D52" r:id="rId31" xr:uid="{7BC6DF64-9FBB-461B-BEE3-D705D5A5711D}"/>
     <hyperlink ref="D21" r:id="rId32" xr:uid="{EE5546A8-9D18-43D6-949A-451AA8A97E76}"/>
-    <hyperlink ref="D73" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
+    <hyperlink ref="D74" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
     <hyperlink ref="D43" r:id="rId34" xr:uid="{03938AC4-898D-4B60-9A83-CF770912371F}"/>
-    <hyperlink ref="D93" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
-    <hyperlink ref="D63" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
+    <hyperlink ref="D94" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
+    <hyperlink ref="D64" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
     <hyperlink ref="D7" r:id="rId37" xr:uid="{C501338A-FD0F-4F45-B8B1-BD737635609F}"/>
     <hyperlink ref="D38" r:id="rId38" xr:uid="{973F790E-4686-49DC-8382-D85663F42FE4}"/>
-    <hyperlink ref="D56" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
-    <hyperlink ref="D95" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
+    <hyperlink ref="D57" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
+    <hyperlink ref="D96" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
     <hyperlink ref="D13" r:id="rId41" xr:uid="{E0321D7C-4A33-425C-AC81-F2844EF49280}"/>
     <hyperlink ref="D45" r:id="rId42" xr:uid="{9362C2F6-92F8-4578-90F4-F93A12DB0620}"/>
     <hyperlink ref="D49" r:id="rId43" xr:uid="{3D2507DB-58F1-46EB-972C-7262C11F3BC0}"/>
     <hyperlink ref="D15" r:id="rId44" xr:uid="{FD7129AB-69C9-448B-90D0-0EB16503D948}"/>
-    <hyperlink ref="D69" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
+    <hyperlink ref="D70" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
     <hyperlink ref="D53" r:id="rId46" xr:uid="{FA35DE19-FE12-4948-8782-601512787A1F}"/>
-    <hyperlink ref="D75" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
-    <hyperlink ref="D81" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
-    <hyperlink ref="D94" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
-    <hyperlink ref="D61" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
+    <hyperlink ref="D76" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
+    <hyperlink ref="D82" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
+    <hyperlink ref="D95" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
+    <hyperlink ref="D62" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
     <hyperlink ref="D27" r:id="rId51" xr:uid="{20CCBF4F-DA07-40B1-84D7-9C64B10A18DD}"/>
     <hyperlink ref="D4" r:id="rId52" xr:uid="{04F40983-3CCF-4A98-9D71-83239E621071}"/>
     <hyperlink ref="D33" r:id="rId53" xr:uid="{B6182D1F-82B7-4DC3-BB62-5D4CE3E6347D}"/>
-    <hyperlink ref="D83" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
-    <hyperlink ref="D101" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
-    <hyperlink ref="D82" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
-    <hyperlink ref="D86" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
+    <hyperlink ref="D84" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
+    <hyperlink ref="D102" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
+    <hyperlink ref="D83" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
+    <hyperlink ref="D87" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
     <hyperlink ref="D9" r:id="rId58" xr:uid="{F7E14BE7-9BEF-429A-BC06-CA914EDCD03E}"/>
     <hyperlink ref="D23" r:id="rId59" xr:uid="{13F0A7EA-4265-4C1A-936D-0F1F22648B66}"/>
     <hyperlink ref="D44" r:id="rId60" display="mailto:david@zwang.com" xr:uid="{2E031ABA-CF1B-48A8-96E6-B6DCE94345AE}"/>
-    <hyperlink ref="D66" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
-    <hyperlink ref="D67" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
-    <hyperlink ref="D89" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
+    <hyperlink ref="D67" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
+    <hyperlink ref="D68" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
+    <hyperlink ref="D90" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
     <hyperlink ref="D30" r:id="rId64" xr:uid="{3AD048BB-9D70-41FA-8645-47CF1BE084C9}"/>
     <hyperlink ref="D32" r:id="rId65" display="mailto:bertvk@enfocus.com" xr:uid="{6F56AFA2-CA54-4A51-B51B-36740F243F7A}"/>
     <hyperlink ref="D47" r:id="rId66" xr:uid="{DEECD580-BF33-4FBB-A267-48E6674FF044}"/>
@@ -4065,7 +4106,7 @@
     <hyperlink ref="D19" r:id="rId68" xr:uid="{897A4DB8-756C-42E5-AF7B-011BBBE00628}"/>
     <hyperlink ref="D40" r:id="rId69" xr:uid="{47A4E692-159B-4E48-A1D4-411E278B3A43}"/>
     <hyperlink ref="D2" r:id="rId70" display="mailto:frank.vyncke@yin4yang.com" xr:uid="{E29600CB-349C-4C55-AC29-3B61912C4757}"/>
-    <hyperlink ref="D100" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
+    <hyperlink ref="D101" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
     <hyperlink ref="D25" r:id="rId72" xr:uid="{BF5FD244-0DE0-493E-A7E1-0CEDCE9B77AA}"/>
     <hyperlink ref="D5" r:id="rId73" xr:uid="{33D12C26-CC5E-4925-86B6-4AE855A6371F}"/>
     <hyperlink ref="G5" r:id="rId74" xr:uid="{2FA39695-7884-42EC-9380-C8EFD7B7EAD9}"/>
@@ -4074,48 +4115,49 @@
     <hyperlink ref="G6" r:id="rId77" xr:uid="{EF6627CA-3B1A-440B-85D4-A1B7067549BD}"/>
     <hyperlink ref="D11" r:id="rId78" xr:uid="{058D1BE7-4CFF-4740-BC92-2074C717A677}"/>
     <hyperlink ref="G11" r:id="rId79" xr:uid="{B9062A46-48F6-45FB-8197-4FD986CC482D}"/>
-    <hyperlink ref="D57" r:id="rId80" xr:uid="{0CFEC845-7F90-4802-9D24-4AC8905CD11B}"/>
-    <hyperlink ref="D64" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
+    <hyperlink ref="D58" r:id="rId80" xr:uid="{0CFEC845-7F90-4802-9D24-4AC8905CD11B}"/>
+    <hyperlink ref="D65" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
     <hyperlink ref="D46" r:id="rId82" xr:uid="{72B2BA10-0B55-4ACF-9CC1-DA30FB4C2741}"/>
     <hyperlink ref="G46" r:id="rId83" xr:uid="{1106BFBB-F6F3-4E8A-8B65-06381130271C}"/>
-    <hyperlink ref="D92" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
-    <hyperlink ref="G92" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
-    <hyperlink ref="G54" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
-    <hyperlink ref="D54" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
+    <hyperlink ref="D93" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
+    <hyperlink ref="G93" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
+    <hyperlink ref="G55" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
+    <hyperlink ref="D55" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
     <hyperlink ref="G20" r:id="rId88" xr:uid="{C64F139E-8286-4E7A-8B5E-9D69FC9A0C25}"/>
-    <hyperlink ref="G60" r:id="rId89" xr:uid="{5D505EE9-2263-469C-9455-D353F4C9921E}"/>
-    <hyperlink ref="D60" r:id="rId90" xr:uid="{5715AC7F-4208-4141-884D-FD2EB9CB5E95}"/>
+    <hyperlink ref="G61" r:id="rId89" xr:uid="{5D505EE9-2263-469C-9455-D353F4C9921E}"/>
+    <hyperlink ref="D61" r:id="rId90" xr:uid="{5715AC7F-4208-4141-884D-FD2EB9CB5E95}"/>
     <hyperlink ref="D18" r:id="rId91" xr:uid="{50E71DF8-A245-41B4-83A8-E6488454D9A4}"/>
     <hyperlink ref="G28" r:id="rId92" xr:uid="{15520162-C027-42E1-8EC1-CA7EA9FD18BC}"/>
     <hyperlink ref="D28" r:id="rId93" xr:uid="{E9A12839-D069-4292-A5EA-36394565B8A0}"/>
     <hyperlink ref="D36" r:id="rId94" xr:uid="{F07464A9-7B4E-4E5B-9EEE-3F687E9DC9AC}"/>
     <hyperlink ref="G36" r:id="rId95" xr:uid="{73C68A69-730D-4676-B564-01BC2FDA7E73}"/>
-    <hyperlink ref="D68" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
-    <hyperlink ref="D99" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
+    <hyperlink ref="D69" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
+    <hyperlink ref="D100" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
     <hyperlink ref="D22" r:id="rId98" xr:uid="{3C768ED5-B6E7-416A-B3CF-31E9B14F1258}"/>
     <hyperlink ref="G22" r:id="rId99" xr:uid="{5C4AC9BE-92AA-40F8-AA34-D54E19486DEE}"/>
     <hyperlink ref="D8" r:id="rId100" xr:uid="{0DDFD3D5-41E0-4A59-8992-A1EE6FD3C05D}"/>
     <hyperlink ref="G8" r:id="rId101" xr:uid="{82F38FA1-9E55-4CDE-87F7-9C87D20D9E51}"/>
-    <hyperlink ref="D74" r:id="rId102" xr:uid="{F47445AD-9EE1-46DB-B7BA-B288E5B3A5E1}"/>
-    <hyperlink ref="G74" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
-    <hyperlink ref="G62" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
-    <hyperlink ref="D62" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
-    <hyperlink ref="D91" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
-    <hyperlink ref="G91" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
-    <hyperlink ref="D55" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
-    <hyperlink ref="G55" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
+    <hyperlink ref="D75" r:id="rId102" xr:uid="{F47445AD-9EE1-46DB-B7BA-B288E5B3A5E1}"/>
+    <hyperlink ref="G75" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
+    <hyperlink ref="G63" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
+    <hyperlink ref="D63" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
+    <hyperlink ref="D92" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
+    <hyperlink ref="G92" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
+    <hyperlink ref="D56" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
+    <hyperlink ref="G56" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
     <hyperlink ref="D24" r:id="rId110" xr:uid="{42EF2DCB-F6A9-4EC5-9C1C-9B9A137FDD6C}"/>
     <hyperlink ref="G24" r:id="rId111" xr:uid="{68016CF6-F4CA-4852-AF56-7954DB739663}"/>
-    <hyperlink ref="D59" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
-    <hyperlink ref="G59" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
-    <hyperlink ref="D79" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
-    <hyperlink ref="G79" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
-    <hyperlink ref="G78" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
+    <hyperlink ref="D60" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
+    <hyperlink ref="G60" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
+    <hyperlink ref="D80" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
+    <hyperlink ref="G80" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
+    <hyperlink ref="G79" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
     <hyperlink ref="D29" r:id="rId117" xr:uid="{B822E1EC-0934-422A-B4A5-1DB34262685E}"/>
-    <hyperlink ref="D71" r:id="rId118" xr:uid="{3ED2EB59-CC97-4952-8CF7-A3B7B8799FDD}"/>
-    <hyperlink ref="G71" r:id="rId119" xr:uid="{D2C2332D-542C-445F-A87F-7165BD629B7F}"/>
+    <hyperlink ref="D72" r:id="rId118" xr:uid="{3ED2EB59-CC97-4952-8CF7-A3B7B8799FDD}"/>
+    <hyperlink ref="G72" r:id="rId119" xr:uid="{D2C2332D-542C-445F-A87F-7165BD629B7F}"/>
+    <hyperlink ref="G54" r:id="rId120" xr:uid="{A59B3571-E2CF-490B-8E2A-49F6F25F2C58}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId120"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId121"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve #57 for NPDF
</commit_message>
<xml_diff>
--- a/ISO PDF Registry.xlsx
+++ b/ISO PDF Registry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\share\pdf-names-list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DFFA40-C60F-4E1F-B436-4EC649609E52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700286B0-03AE-4A09-BE11-0030F4D6B708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3456" yWindow="3456" windowWidth="21600" windowHeight="13560" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
+    <workbookView xWindow="-26430" yWindow="2130" windowWidth="21600" windowHeight="13560" tabRatio="536" xr2:uid="{9E3ABFD2-C7ED-CB44-90E8-944996B24765}"/>
   </bookViews>
   <sheets>
     <sheet name="PDF Prefix Registry" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="484">
   <si>
     <t>ITXT</t>
   </si>
@@ -1464,6 +1464,24 @@
   </si>
   <si>
     <t>Christian.Nyffenegger@linkgenetic.com</t>
+  </si>
+  <si>
+    <t>NPDF</t>
+  </si>
+  <si>
+    <t>Jerry</t>
+  </si>
+  <si>
+    <t>Wang</t>
+  </si>
+  <si>
+    <t>support@getnextpdf.com</t>
+  </si>
+  <si>
+    <t>PATEON Network Technology Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/adobe/pdf-names-list/issues/57 </t>
   </si>
 </sst>
 </file>
@@ -1887,7 +1905,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E74889-C943-2949-BDAA-069F646F779D}">
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" customWidth="1"/>
@@ -3287,27 +3305,30 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>282</v>
+        <v>478</v>
       </c>
       <c r="B67" t="s">
-        <v>285</v>
+        <v>479</v>
       </c>
       <c r="C67" t="s">
-        <v>286</v>
+        <v>480</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>287</v>
+        <v>481</v>
       </c>
       <c r="E67" t="s">
-        <v>284</v>
+        <v>482</v>
       </c>
       <c r="F67" s="5">
-        <v>44580</v>
+        <v>46227</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>483</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B68" t="s">
         <v>285</v>
@@ -3327,90 +3348,87 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>408</v>
+        <v>283</v>
       </c>
       <c r="B69" t="s">
-        <v>361</v>
+        <v>285</v>
       </c>
       <c r="C69" t="s">
-        <v>362</v>
+        <v>286</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>363</v>
+        <v>287</v>
       </c>
       <c r="E69" t="s">
-        <v>214</v>
+        <v>284</v>
       </c>
       <c r="F69" s="5">
-        <v>45695</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>89</v>
+        <v>408</v>
       </c>
       <c r="B70" t="s">
-        <v>90</v>
+        <v>361</v>
       </c>
       <c r="C70" t="s">
-        <v>91</v>
+        <v>362</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>92</v>
+        <v>363</v>
       </c>
       <c r="E70" t="s">
-        <v>93</v>
+        <v>214</v>
       </c>
       <c r="F70" s="5">
-        <v>41780</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>161</v>
+        <v>89</v>
       </c>
       <c r="B71" t="s">
-        <v>162</v>
+        <v>90</v>
       </c>
       <c r="C71" t="s">
-        <v>163</v>
+        <v>91</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>164</v>
+        <v>92</v>
       </c>
       <c r="E71" t="s">
-        <v>165</v>
+        <v>93</v>
       </c>
       <c r="F71" s="5">
-        <v>42530</v>
+        <v>41780</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>469</v>
+        <v>161</v>
       </c>
       <c r="B72" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="C72" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>122</v>
+        <v>164</v>
       </c>
       <c r="E72" t="s">
-        <v>214</v>
+        <v>165</v>
       </c>
       <c r="F72" s="5">
-        <v>46147</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>470</v>
+        <v>42530</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>213</v>
+        <v>469</v>
       </c>
       <c r="B73" t="s">
         <v>120</v>
@@ -3425,490 +3443,493 @@
         <v>214</v>
       </c>
       <c r="F73" s="5">
-        <v>43502</v>
-      </c>
-      <c r="G73" t="s">
-        <v>471</v>
+        <v>46147</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>29</v>
+        <v>213</v>
       </c>
       <c r="B74" t="s">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="C74" t="s">
-        <v>31</v>
+        <v>121</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="E74" t="s">
-        <v>33</v>
+        <v>214</v>
       </c>
       <c r="F74" s="5">
-        <v>40164.4375</v>
+        <v>43502</v>
+      </c>
+      <c r="G74" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>423</v>
+        <v>29</v>
       </c>
       <c r="B75" t="s">
-        <v>424</v>
+        <v>30</v>
       </c>
       <c r="C75" t="s">
-        <v>425</v>
+        <v>31</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>426</v>
+        <v>32</v>
+      </c>
+      <c r="E75" t="s">
+        <v>33</v>
       </c>
       <c r="F75" s="5">
-        <v>45803</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>427</v>
+        <v>40164.4375</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>99</v>
+        <v>423</v>
       </c>
       <c r="B76" t="s">
-        <v>100</v>
+        <v>424</v>
       </c>
       <c r="C76" t="s">
-        <v>101</v>
+        <v>425</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E76" t="s">
-        <v>103</v>
+        <v>426</v>
       </c>
       <c r="F76" s="5">
-        <v>41854</v>
+        <v>45803</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
+        <v>99</v>
+      </c>
+      <c r="B77" t="s">
+        <v>100</v>
+      </c>
+      <c r="C77" t="s">
+        <v>101</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E77" t="s">
+        <v>103</v>
+      </c>
+      <c r="F77" s="5">
+        <v>41854</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
         <v>198</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B78" t="s">
         <v>199</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C78" t="s">
         <v>200</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="D78" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="E77" s="5" t="s">
+      <c r="E78" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="F77" s="6">
+      <c r="F78" s="6">
         <v>37415</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="C78" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="E78" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="F78" s="5">
-        <v>43997</v>
-      </c>
-      <c r="G78" s="7" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="7" t="s">
-        <v>460</v>
+        <v>238</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="C79" t="s">
-        <v>462</v>
+        <v>234</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>235</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="E79" t="s">
-        <v>464</v>
+        <v>236</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>237</v>
       </c>
       <c r="F79" s="5">
-        <v>46090</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>465</v>
+        <v>43997</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>441</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="C80" t="s">
+        <v>462</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="E80" t="s">
+        <v>464</v>
+      </c>
+      <c r="F80" s="5">
+        <v>46090</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="B81" s="7" t="s">
         <v>455</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="C81" s="7" t="s">
         <v>456</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="D81" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E80" s="7" t="s">
+      <c r="E81" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="F80" s="5">
+      <c r="F81" s="5">
         <v>46038</v>
       </c>
-      <c r="G80" s="1" t="s">
+      <c r="G81" s="1" t="s">
         <v>459</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>253</v>
-      </c>
-      <c r="B81" t="s">
-        <v>254</v>
-      </c>
-      <c r="C81" t="s">
-        <v>255</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E81" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="F81" s="5">
-        <v>44166</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>104</v>
+        <v>253</v>
       </c>
       <c r="B82" t="s">
-        <v>105</v>
+        <v>254</v>
       </c>
       <c r="C82" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E82" t="s">
-        <v>108</v>
+        <v>256</v>
+      </c>
+      <c r="E82" s="8" t="s">
+        <v>257</v>
       </c>
       <c r="F82" s="5">
-        <v>41857</v>
+        <v>44166</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="B83" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="C83" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>146</v>
+        <v>107</v>
       </c>
       <c r="E83" t="s">
-        <v>147</v>
+        <v>108</v>
       </c>
       <c r="F83" s="5">
-        <v>42467</v>
+        <v>41857</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B84" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C84" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E84" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="F84" s="5">
-        <v>42420</v>
+        <v>42467</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>227</v>
+        <v>133</v>
       </c>
       <c r="B85" t="s">
-        <v>228</v>
+        <v>134</v>
       </c>
       <c r="C85" t="s">
-        <v>229</v>
+        <v>135</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>230</v>
+        <v>136</v>
       </c>
       <c r="E85" t="s">
-        <v>231</v>
+        <v>137</v>
       </c>
       <c r="F85" s="5">
-        <v>43973</v>
+        <v>42420</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="B86" t="s">
-        <v>15</v>
+        <v>228</v>
       </c>
       <c r="C86" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="E86" t="s">
-        <v>18</v>
+        <v>231</v>
       </c>
       <c r="F86" s="5">
-        <v>40081.550694444442</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>148</v>
+        <v>14</v>
       </c>
       <c r="B87" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C87" t="s">
-        <v>149</v>
+        <v>16</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="E87" t="s">
-        <v>151</v>
+        <v>18</v>
       </c>
       <c r="F87" s="5">
-        <v>42472</v>
+        <v>40081.550694444442</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="B88" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C88" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="E88" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
       <c r="F88" s="5">
-        <v>43054</v>
+        <v>42472</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="B89" t="s">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="C89" t="s">
-        <v>301</v>
+        <v>179</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="E89" t="s">
-        <v>221</v>
+        <v>181</v>
       </c>
       <c r="F89" s="5">
-        <v>43973</v>
+        <v>43054</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="B90" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="C90" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>290</v>
+        <v>220</v>
       </c>
       <c r="E90" t="s">
-        <v>289</v>
+        <v>221</v>
       </c>
       <c r="F90" s="5">
-        <v>44580</v>
+        <v>43973</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>172</v>
+        <v>288</v>
       </c>
       <c r="B91" t="s">
-        <v>173</v>
+        <v>291</v>
       </c>
       <c r="C91" t="s">
-        <v>174</v>
+        <v>292</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>175</v>
+        <v>290</v>
       </c>
       <c r="E91" t="s">
-        <v>176</v>
+        <v>289</v>
       </c>
       <c r="F91" s="5">
-        <v>42739</v>
+        <v>44580</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>431</v>
+        <v>172</v>
       </c>
       <c r="B92" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C92" t="s">
-        <v>432</v>
+        <v>174</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>433</v>
+        <v>175</v>
       </c>
       <c r="E92" t="s">
-        <v>434</v>
+        <v>176</v>
       </c>
       <c r="F92" s="5">
-        <v>45818</v>
-      </c>
-      <c r="G92" s="1" t="s">
-        <v>435</v>
+        <v>42739</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>375</v>
+        <v>431</v>
       </c>
       <c r="B93" t="s">
-        <v>376</v>
+        <v>183</v>
       </c>
       <c r="C93" t="s">
-        <v>377</v>
+        <v>432</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="E93" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="F93" s="5">
-        <v>45358</v>
+        <v>45818</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>39</v>
+        <v>375</v>
       </c>
       <c r="B94" t="s">
-        <v>40</v>
+        <v>376</v>
       </c>
       <c r="C94" t="s">
-        <v>41</v>
+        <v>377</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>42</v>
+        <v>378</v>
       </c>
       <c r="E94" t="s">
-        <v>43</v>
+        <v>379</v>
       </c>
       <c r="F94" s="5">
-        <v>40522.519444444442</v>
+        <v>45358</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="B95" t="s">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="C95" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="E95" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="F95" s="5">
-        <v>41890</v>
+        <v>40522.519444444442</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="B96" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="C96" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="E96" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="F96" s="5">
-        <v>42852</v>
+        <v>41890</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>177</v>
+        <v>64</v>
       </c>
       <c r="B97" t="s">
         <v>65</v>
@@ -3928,104 +3949,124 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B98" t="s">
-        <v>204</v>
+        <v>65</v>
       </c>
       <c r="C98" t="s">
-        <v>205</v>
+        <v>66</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="F98" s="6">
-        <v>43487</v>
+        <v>67</v>
+      </c>
+      <c r="E98" t="s">
+        <v>68</v>
+      </c>
+      <c r="F98" s="5">
+        <v>42852</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="B99" t="s">
-        <v>157</v>
+        <v>204</v>
       </c>
       <c r="C99" t="s">
-        <v>158</v>
+        <v>205</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E99" t="s">
-        <v>160</v>
-      </c>
-      <c r="F99" s="5">
-        <v>42505</v>
+        <v>206</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F99" s="6">
+        <v>43487</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>409</v>
+        <v>156</v>
       </c>
       <c r="B100" t="s">
-        <v>361</v>
+        <v>157</v>
       </c>
       <c r="C100" t="s">
-        <v>362</v>
+        <v>158</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>363</v>
+        <v>159</v>
       </c>
       <c r="E100" t="s">
-        <v>214</v>
+        <v>160</v>
       </c>
       <c r="F100" s="5">
-        <v>45695</v>
-      </c>
-      <c r="G100" t="s">
-        <v>410</v>
+        <v>42505</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>329</v>
+        <v>409</v>
       </c>
       <c r="B101" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C101" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="E101" t="s">
-        <v>333</v>
+        <v>214</v>
       </c>
       <c r="F101" s="5">
-        <v>44775</v>
+        <v>45695</v>
+      </c>
+      <c r="G101" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
+        <v>329</v>
+      </c>
+      <c r="B102" t="s">
+        <v>330</v>
+      </c>
+      <c r="C102" t="s">
+        <v>331</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E102" t="s">
+        <v>333</v>
+      </c>
+      <c r="F102" s="5">
+        <v>44775</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
         <v>138</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B103" t="s">
         <v>139</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C103" t="s">
         <v>140</v>
       </c>
-      <c r="D102" s="1" t="s">
+      <c r="D103" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E102" t="s">
+      <c r="E103" t="s">
         <v>142</v>
       </c>
-      <c r="F102" s="5">
+      <c r="F103" s="5">
         <v>42439</v>
       </c>
     </row>
@@ -4037,68 +4078,68 @@
   </autoFilter>
   <hyperlinks>
     <hyperlink ref="D66" r:id="rId1" xr:uid="{407FC650-7151-6940-B8FA-60477C7D30B1}"/>
-    <hyperlink ref="D73" r:id="rId2" xr:uid="{68E4476D-88C7-5D40-9274-7B03AB299562}"/>
+    <hyperlink ref="D74" r:id="rId2" xr:uid="{68E4476D-88C7-5D40-9274-7B03AB299562}"/>
     <hyperlink ref="D59" r:id="rId3" display="mailto:klink@csi.com" xr:uid="{85C07C9E-BB28-4C49-84D2-B3052E15F688}"/>
     <hyperlink ref="D50" r:id="rId4" xr:uid="{234AD513-3ABE-F545-A037-27824EABDF68}"/>
     <hyperlink ref="D42" r:id="rId5" xr:uid="{7924D455-5B5F-E641-AB7C-FB4BD03EF051}"/>
-    <hyperlink ref="D85" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
+    <hyperlink ref="D86" r:id="rId6" display="mailto:normand.williams@onespan.com" xr:uid="{C8F08AEB-A945-364E-84E9-3EFCB37949EA}"/>
     <hyperlink ref="D41" r:id="rId7" xr:uid="{7AEF03BC-D893-FF42-BB52-AB9C9480EA0D}"/>
-    <hyperlink ref="D89" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
+    <hyperlink ref="D90" r:id="rId8" xr:uid="{1E7EE29B-6F34-AF43-9A6A-A4BA495EE964}"/>
     <hyperlink ref="D12" r:id="rId9" xr:uid="{D57F2423-845A-9E44-A60D-DEEB1150BE7A}"/>
     <hyperlink ref="D10" r:id="rId10" xr:uid="{0133BED0-2D2B-4A0F-AB7C-D58D8B5F381B}"/>
     <hyperlink ref="D3" r:id="rId11" xr:uid="{5F0875F3-1434-4B08-A87A-2BDF5EEDDAC9}"/>
     <hyperlink ref="D26" r:id="rId12" xr:uid="{61482C13-D6B2-4AFF-AD10-908ABE8BA3F2}"/>
-    <hyperlink ref="D81" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
+    <hyperlink ref="D82" r:id="rId13" xr:uid="{8AA40E15-5F88-4955-98D8-3EDB9CE3C08B}"/>
     <hyperlink ref="D48" r:id="rId14" xr:uid="{FEB07F00-70C8-4D84-B7DF-B36DF7C6138C}"/>
     <hyperlink ref="D37" r:id="rId15" xr:uid="{9236AFAC-B489-4804-B65A-1988399CC4C2}"/>
-    <hyperlink ref="D78" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
-    <hyperlink ref="D98" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
-    <hyperlink ref="D77" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
+    <hyperlink ref="D79" r:id="rId16" xr:uid="{50BFEC84-47AF-4D28-B04F-52D949215BCB}"/>
+    <hyperlink ref="D99" r:id="rId17" xr:uid="{29C24CB5-B24B-4772-A291-FC2CDC7AB656}"/>
+    <hyperlink ref="D78" r:id="rId18" xr:uid="{6A8074F9-38E6-46D2-BC30-EDB597684655}"/>
     <hyperlink ref="D31" r:id="rId19" xr:uid="{178F076F-6CAC-44EB-AA97-31037608AA41}"/>
     <hyperlink ref="D39" r:id="rId20" xr:uid="{E467E97B-65A6-40E0-A2BA-7875E3A5C2C1}"/>
-    <hyperlink ref="D88" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
-    <hyperlink ref="D97" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
-    <hyperlink ref="D91" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
+    <hyperlink ref="D89" r:id="rId21" xr:uid="{6177B640-2E3A-4478-8CB7-5ED41AA4BC0A}"/>
+    <hyperlink ref="D98" r:id="rId22" xr:uid="{51676D7C-EE2B-463D-8301-98CF22D9B71E}"/>
+    <hyperlink ref="D92" r:id="rId23" xr:uid="{DB05FA17-E2C3-49C9-8F48-C3395EC9FB65}"/>
     <hyperlink ref="D17" r:id="rId24" xr:uid="{8C069B77-F7A2-4DC6-9D5A-D5138E5E1158}"/>
     <hyperlink ref="D16" r:id="rId25" xr:uid="{C770D7DE-6980-45A2-A8B6-8E4C376C05E3}"/>
-    <hyperlink ref="D71" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
-    <hyperlink ref="D99" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
+    <hyperlink ref="D72" r:id="rId26" xr:uid="{17A234E9-7249-4FCC-8BD4-B42E6DD51533}"/>
+    <hyperlink ref="D100" r:id="rId27" xr:uid="{B26FB768-9814-44C0-BE49-D50110CF8838}"/>
     <hyperlink ref="D51" r:id="rId28" xr:uid="{2B927B9E-56D2-4AC7-A24B-BA7FAF44F900}"/>
     <hyperlink ref="D34" r:id="rId29" xr:uid="{5F9DAD98-7221-4BEC-B311-BF6B1BD6F52E}"/>
-    <hyperlink ref="D86" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
+    <hyperlink ref="D87" r:id="rId30" xr:uid="{9388EE39-1B30-49DB-89AC-BEC39E8ACFBE}"/>
     <hyperlink ref="D52" r:id="rId31" xr:uid="{7BC6DF64-9FBB-461B-BEE3-D705D5A5711D}"/>
     <hyperlink ref="D21" r:id="rId32" xr:uid="{EE5546A8-9D18-43D6-949A-451AA8A97E76}"/>
-    <hyperlink ref="D74" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
+    <hyperlink ref="D75" r:id="rId33" xr:uid="{02A107CB-A6C9-40AA-AF84-5B08D008A43D}"/>
     <hyperlink ref="D43" r:id="rId34" xr:uid="{03938AC4-898D-4B60-9A83-CF770912371F}"/>
-    <hyperlink ref="D94" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
+    <hyperlink ref="D95" r:id="rId35" xr:uid="{3EECDB74-289B-411A-BCC5-A028AA2ED5D5}"/>
     <hyperlink ref="D64" r:id="rId36" xr:uid="{DEE2DB12-0D3D-4E58-8948-C29EDF524684}"/>
     <hyperlink ref="D7" r:id="rId37" xr:uid="{C501338A-FD0F-4F45-B8B1-BD737635609F}"/>
     <hyperlink ref="D38" r:id="rId38" xr:uid="{973F790E-4686-49DC-8382-D85663F42FE4}"/>
     <hyperlink ref="D57" r:id="rId39" xr:uid="{EB649DE9-649F-4972-9591-B77A8EC85DED}"/>
-    <hyperlink ref="D96" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
+    <hyperlink ref="D97" r:id="rId40" xr:uid="{381C8997-BEB8-4BF6-B715-C9CE36B18767}"/>
     <hyperlink ref="D13" r:id="rId41" xr:uid="{E0321D7C-4A33-425C-AC81-F2844EF49280}"/>
     <hyperlink ref="D45" r:id="rId42" xr:uid="{9362C2F6-92F8-4578-90F4-F93A12DB0620}"/>
     <hyperlink ref="D49" r:id="rId43" xr:uid="{3D2507DB-58F1-46EB-972C-7262C11F3BC0}"/>
     <hyperlink ref="D15" r:id="rId44" xr:uid="{FD7129AB-69C9-448B-90D0-0EB16503D948}"/>
-    <hyperlink ref="D70" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
+    <hyperlink ref="D71" r:id="rId45" xr:uid="{4F9A8AB7-9ABA-4133-A103-EC20BB3D5255}"/>
     <hyperlink ref="D53" r:id="rId46" xr:uid="{FA35DE19-FE12-4948-8782-601512787A1F}"/>
-    <hyperlink ref="D76" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
-    <hyperlink ref="D82" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
-    <hyperlink ref="D95" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
+    <hyperlink ref="D77" r:id="rId47" xr:uid="{150BA8A8-C8E4-466E-B635-B3C8D844E311}"/>
+    <hyperlink ref="D83" r:id="rId48" xr:uid="{9D9D1EDB-1408-4DC1-94C7-2F6827AB67F5}"/>
+    <hyperlink ref="D96" r:id="rId49" xr:uid="{EB91F0BD-5E69-461C-9E7C-D329942BCBBE}"/>
     <hyperlink ref="D62" r:id="rId50" xr:uid="{1D2CC020-5555-4E5F-87C1-5B10ECF5CEE5}"/>
     <hyperlink ref="D27" r:id="rId51" xr:uid="{20CCBF4F-DA07-40B1-84D7-9C64B10A18DD}"/>
     <hyperlink ref="D4" r:id="rId52" xr:uid="{04F40983-3CCF-4A98-9D71-83239E621071}"/>
     <hyperlink ref="D33" r:id="rId53" xr:uid="{B6182D1F-82B7-4DC3-BB62-5D4CE3E6347D}"/>
-    <hyperlink ref="D84" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
-    <hyperlink ref="D102" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
-    <hyperlink ref="D83" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
-    <hyperlink ref="D87" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
+    <hyperlink ref="D85" r:id="rId54" xr:uid="{7F7DBD18-50DD-4284-8836-015BE6E2AF57}"/>
+    <hyperlink ref="D103" r:id="rId55" xr:uid="{2160B5D2-BA90-4A96-B73C-39ADAF82E7EC}"/>
+    <hyperlink ref="D84" r:id="rId56" xr:uid="{35C5AF31-961F-47D5-AF98-5D77E6CC3905}"/>
+    <hyperlink ref="D88" r:id="rId57" xr:uid="{3776AFCD-5853-4CE7-A817-305F74165C06}"/>
     <hyperlink ref="D9" r:id="rId58" xr:uid="{F7E14BE7-9BEF-429A-BC06-CA914EDCD03E}"/>
     <hyperlink ref="D23" r:id="rId59" xr:uid="{13F0A7EA-4265-4C1A-936D-0F1F22648B66}"/>
     <hyperlink ref="D44" r:id="rId60" display="mailto:david@zwang.com" xr:uid="{2E031ABA-CF1B-48A8-96E6-B6DCE94345AE}"/>
-    <hyperlink ref="D67" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
-    <hyperlink ref="D68" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
-    <hyperlink ref="D90" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
+    <hyperlink ref="D68" r:id="rId61" xr:uid="{1245116C-C3B7-4F34-8A1E-A3AF6A558128}"/>
+    <hyperlink ref="D69" r:id="rId62" xr:uid="{DF5F6B9A-45BB-416F-8E3D-91269D73D457}"/>
+    <hyperlink ref="D91" r:id="rId63" xr:uid="{E4C2E6D9-1E4B-4B0D-8600-86E3ECB7D1D8}"/>
     <hyperlink ref="D30" r:id="rId64" xr:uid="{3AD048BB-9D70-41FA-8645-47CF1BE084C9}"/>
     <hyperlink ref="D32" r:id="rId65" display="mailto:bertvk@enfocus.com" xr:uid="{6F56AFA2-CA54-4A51-B51B-36740F243F7A}"/>
     <hyperlink ref="D47" r:id="rId66" xr:uid="{DEECD580-BF33-4FBB-A267-48E6674FF044}"/>
@@ -4106,7 +4147,7 @@
     <hyperlink ref="D19" r:id="rId68" xr:uid="{897A4DB8-756C-42E5-AF7B-011BBBE00628}"/>
     <hyperlink ref="D40" r:id="rId69" xr:uid="{47A4E692-159B-4E48-A1D4-411E278B3A43}"/>
     <hyperlink ref="D2" r:id="rId70" display="mailto:frank.vyncke@yin4yang.com" xr:uid="{E29600CB-349C-4C55-AC29-3B61912C4757}"/>
-    <hyperlink ref="D101" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
+    <hyperlink ref="D102" r:id="rId71" xr:uid="{C4C4EA22-387A-4AD7-A4B4-D79D02B39793}"/>
     <hyperlink ref="D25" r:id="rId72" xr:uid="{BF5FD244-0DE0-493E-A7E1-0CEDCE9B77AA}"/>
     <hyperlink ref="D5" r:id="rId73" xr:uid="{33D12C26-CC5E-4925-86B6-4AE855A6371F}"/>
     <hyperlink ref="G5" r:id="rId74" xr:uid="{2FA39695-7884-42EC-9380-C8EFD7B7EAD9}"/>
@@ -4119,8 +4160,8 @@
     <hyperlink ref="D65" r:id="rId81" xr:uid="{81B44739-2F1A-4DDB-90E8-2523712052F0}"/>
     <hyperlink ref="D46" r:id="rId82" xr:uid="{72B2BA10-0B55-4ACF-9CC1-DA30FB4C2741}"/>
     <hyperlink ref="G46" r:id="rId83" xr:uid="{1106BFBB-F6F3-4E8A-8B65-06381130271C}"/>
-    <hyperlink ref="D93" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
-    <hyperlink ref="G93" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
+    <hyperlink ref="D94" r:id="rId84" xr:uid="{249742DB-9523-4D5C-B3FC-194F7D7BB889}"/>
+    <hyperlink ref="G94" r:id="rId85" xr:uid="{BD0ABADB-115E-43D9-8791-2BFF7CAEC355}"/>
     <hyperlink ref="G55" r:id="rId86" xr:uid="{44657DD4-3FFA-4E6F-8898-631518A1BFDC}"/>
     <hyperlink ref="D55" r:id="rId87" xr:uid="{D5A339A1-161D-40E3-9F69-B4599246184B}"/>
     <hyperlink ref="G20" r:id="rId88" xr:uid="{C64F139E-8286-4E7A-8B5E-9D69FC9A0C25}"/>
@@ -4131,33 +4172,35 @@
     <hyperlink ref="D28" r:id="rId93" xr:uid="{E9A12839-D069-4292-A5EA-36394565B8A0}"/>
     <hyperlink ref="D36" r:id="rId94" xr:uid="{F07464A9-7B4E-4E5B-9EEE-3F687E9DC9AC}"/>
     <hyperlink ref="G36" r:id="rId95" xr:uid="{73C68A69-730D-4676-B564-01BC2FDA7E73}"/>
-    <hyperlink ref="D69" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
-    <hyperlink ref="D100" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
+    <hyperlink ref="D70" r:id="rId96" xr:uid="{DC40AB03-35C7-4C6E-B261-5A4793D79E6C}"/>
+    <hyperlink ref="D101" r:id="rId97" xr:uid="{474ED1A8-8C48-45EA-B1FF-F6F7564A2191}"/>
     <hyperlink ref="D22" r:id="rId98" xr:uid="{3C768ED5-B6E7-416A-B3CF-31E9B14F1258}"/>
     <hyperlink ref="G22" r:id="rId99" xr:uid="{5C4AC9BE-92AA-40F8-AA34-D54E19486DEE}"/>
     <hyperlink ref="D8" r:id="rId100" xr:uid="{0DDFD3D5-41E0-4A59-8992-A1EE6FD3C05D}"/>
     <hyperlink ref="G8" r:id="rId101" xr:uid="{82F38FA1-9E55-4CDE-87F7-9C87D20D9E51}"/>
-    <hyperlink ref="D75" r:id="rId102" xr:uid="{F47445AD-9EE1-46DB-B7BA-B288E5B3A5E1}"/>
-    <hyperlink ref="G75" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
+    <hyperlink ref="D76" r:id="rId102" xr:uid="{F47445AD-9EE1-46DB-B7BA-B288E5B3A5E1}"/>
+    <hyperlink ref="G76" r:id="rId103" xr:uid="{E84E1C75-8DAE-4F16-81A7-9CFD148DB33C}"/>
     <hyperlink ref="G63" r:id="rId104" xr:uid="{F4B6441E-03BA-4590-A037-2716147A1E52}"/>
     <hyperlink ref="D63" r:id="rId105" xr:uid="{06F67F32-1CA6-4040-9EE9-F5DDCC803FD8}"/>
-    <hyperlink ref="D92" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
-    <hyperlink ref="G92" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
+    <hyperlink ref="D93" r:id="rId106" xr:uid="{73290877-BE70-4142-A675-1B6E6DA9A816}"/>
+    <hyperlink ref="G93" r:id="rId107" xr:uid="{98760A92-F2C2-4C4B-9C7E-F5B45E828D56}"/>
     <hyperlink ref="D56" r:id="rId108" display="mailto:latex-team@latex-project.org" xr:uid="{2D1B71BC-D0DA-42EA-A440-B30893B690F6}"/>
     <hyperlink ref="G56" r:id="rId109" xr:uid="{6FE50AE6-B4B4-4755-B413-4A3EBE471F2F}"/>
     <hyperlink ref="D24" r:id="rId110" xr:uid="{42EF2DCB-F6A9-4EC5-9C1C-9B9A137FDD6C}"/>
     <hyperlink ref="G24" r:id="rId111" xr:uid="{68016CF6-F4CA-4852-AF56-7954DB739663}"/>
     <hyperlink ref="D60" r:id="rId112" xr:uid="{2C048A18-E375-47C9-B949-DFA2CD2A49F7}"/>
     <hyperlink ref="G60" r:id="rId113" xr:uid="{52F53FAB-AE36-4CDA-BCD8-79975803A89F}"/>
-    <hyperlink ref="D80" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
-    <hyperlink ref="G80" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
-    <hyperlink ref="G79" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
+    <hyperlink ref="D81" r:id="rId114" xr:uid="{C07D46B8-E47D-483E-A1D9-1B4120FCDE06}"/>
+    <hyperlink ref="G81" r:id="rId115" xr:uid="{8A116893-F309-40AA-98CF-5D3145C29816}"/>
+    <hyperlink ref="G80" r:id="rId116" xr:uid="{52643863-FFC9-43C1-BACB-DCB9FD7B4B2D}"/>
     <hyperlink ref="D29" r:id="rId117" xr:uid="{B822E1EC-0934-422A-B4A5-1DB34262685E}"/>
-    <hyperlink ref="D72" r:id="rId118" xr:uid="{3ED2EB59-CC97-4952-8CF7-A3B7B8799FDD}"/>
-    <hyperlink ref="G72" r:id="rId119" xr:uid="{D2C2332D-542C-445F-A87F-7165BD629B7F}"/>
+    <hyperlink ref="D73" r:id="rId118" xr:uid="{3ED2EB59-CC97-4952-8CF7-A3B7B8799FDD}"/>
+    <hyperlink ref="G73" r:id="rId119" xr:uid="{D2C2332D-542C-445F-A87F-7165BD629B7F}"/>
     <hyperlink ref="G54" r:id="rId120" xr:uid="{A59B3571-E2CF-490B-8E2A-49F6F25F2C58}"/>
+    <hyperlink ref="D67" r:id="rId121" xr:uid="{7C2A90B1-2C07-495B-B90B-ABFCB03EC3B2}"/>
+    <hyperlink ref="G67" r:id="rId122" xr:uid="{F8171A08-DE7F-4E75-B92E-3D3692A27AE6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId121"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId123"/>
 </worksheet>
 </file>
</xml_diff>